<commit_message>
Consumibles: lija en rollo por metro, aviso de unidad en Catálogo y limpieza del repo
- La lija en rollo de 45 m (#36 a #100) se entrega cortada: unidad metro,
  compra por rollo de 45 y costo por metro. El retiro del 13/10 que figuraba
  como 2 rollos ($287.812) se anuló y se volvió a cargar como 2 metros.
  Migración 20261013180000, ya aplicada.
- Catálogo: filtro "Revisar unidad" y aviso en la ficha para blísteres,
  rollos que se cortan y cajas por N con la unidad en "una" (regla
  motivoRevisarUnidad con su prueba).
- Excel de consumo regenerado con el registro corregido.
- Fuera del repo (siguen en disco): outputs/ de los agentes (perfiles de
  Chrome, driver de la impresora, planillas de prueba y archivos de bloqueo
  de Office) y el estado local de .claude-flow, que ya estaba en .gitignore.
  Se suman outputs/ y ~$* al .gitignore.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entregables/consumibles/consumo-consumibles-2026-10-13.xlsx
+++ b/entregables/consumibles/consumo-consumibles-2026-10-13.xlsx
@@ -23,7 +23,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6">'Por mes y rubro'!$A$1:$D$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7">'Por producto'!$A$1:$H$141</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8">'Sin valorizar'!$A$1:$E$43</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9">'Registro nuevo (desde 13-10)'!$A$1:$P$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9">'Registro nuevo (desde 13-10)'!$A$1:$P$98</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -497,7 +497,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P10"/>
+  <dimension ref="A1:P98"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="7.83203125" customWidth="1"/>
@@ -596,25 +596,25 @@
         <v>Chubut</v>
       </c>
       <c r="J2" t="str">
-        <v>Cinta papel DobleA VERDE 48mm</v>
+        <v>Lija en rollo 0,12x45mts #36</v>
       </c>
       <c r="K2" t="str">
-        <v>C0032</v>
+        <v>L0037</v>
       </c>
       <c r="L2" s="1">
         <v>2</v>
       </c>
       <c r="M2" t="str">
-        <v>rollo</v>
+        <v>metro</v>
       </c>
       <c r="N2" s="2">
-        <v>5287.36</v>
+        <v>3197.9141</v>
       </c>
       <c r="O2" s="2">
-        <v>10574.72</v>
+        <v>6395.83</v>
       </c>
       <c r="P2" t="str">
-        <v/>
+        <v>Recargado en metros (figuraba en rollos de 45 m)</v>
       </c>
     </row>
     <row r="3">
@@ -646,10 +646,10 @@
         <v>Chubut</v>
       </c>
       <c r="J3" t="str">
-        <v>Lija en rollo 0,12x45mts #36</v>
+        <v>Cinta papel DobleA VERDE 48mm</v>
       </c>
       <c r="K3" t="str">
-        <v>L0037</v>
+        <v>C0032</v>
       </c>
       <c r="L3" s="1">
         <v>2</v>
@@ -658,10 +658,10 @@
         <v>rollo</v>
       </c>
       <c r="N3" s="2">
-        <v>143906.1363</v>
+        <v>5287.36</v>
       </c>
       <c r="O3" s="2">
-        <v>287812.27</v>
+        <v>10574.72</v>
       </c>
       <c r="P3" t="str">
         <v/>
@@ -1017,10 +1017,4410 @@
         <v/>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B11" t="str">
+        <v>09:00 a. m.</v>
+      </c>
+      <c r="C11" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D11" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Ruiz Ernan Eleuterio</v>
+      </c>
+      <c r="F11" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G11" t="str">
+        <v>55-3</v>
+      </c>
+      <c r="H11" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I11" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J11" t="str">
+        <v>LIJA IMPORTADA NO PAST #320</v>
+      </c>
+      <c r="K11" t="str">
+        <v>L0070</v>
+      </c>
+      <c r="L11" s="1">
+        <v>10</v>
+      </c>
+      <c r="M11" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N11" s="2">
+        <v>539</v>
+      </c>
+      <c r="O11" s="2">
+        <v>5390</v>
+      </c>
+      <c r="P11" t="str">
+        <v>Solicitud N° 197</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B12" t="str">
+        <v>09:00 a. m.</v>
+      </c>
+      <c r="C12" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D12" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Ruiz Ernan Eleuterio</v>
+      </c>
+      <c r="F12" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G12" t="str">
+        <v>55-3</v>
+      </c>
+      <c r="H12" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I12" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J12" t="str">
+        <v>Trapo Blanco CAMISETA x Kilo</v>
+      </c>
+      <c r="K12" t="str">
+        <v>T0009</v>
+      </c>
+      <c r="L12" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="M12" t="str">
+        <v>kg</v>
+      </c>
+      <c r="N12" s="2">
+        <v>3280</v>
+      </c>
+      <c r="O12" s="2">
+        <v>1640</v>
+      </c>
+      <c r="P12" t="str">
+        <v>Solicitud N° 197</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B13" t="str">
+        <v>09:00 a. m.</v>
+      </c>
+      <c r="C13" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D13" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Ruiz Ernan Eleuterio</v>
+      </c>
+      <c r="F13" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G13" t="str">
+        <v>55-3</v>
+      </c>
+      <c r="H13" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I13" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J13" t="str">
+        <v>LIJA A/AGUA AA MICROGRANO#2000</v>
+      </c>
+      <c r="K13" t="str">
+        <v>L0023</v>
+      </c>
+      <c r="L13" s="1">
+        <v>10</v>
+      </c>
+      <c r="M13" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N13" s="2">
+        <v>1334.9292</v>
+      </c>
+      <c r="O13" s="2">
+        <v>13349.29</v>
+      </c>
+      <c r="P13" t="str">
+        <v>Solicitud N° 197</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B14" t="str">
+        <v>09:00 a. m.</v>
+      </c>
+      <c r="C14" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D14" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Ruiz Ernan Eleuterio</v>
+      </c>
+      <c r="F14" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G14" t="str">
+        <v>55-3</v>
+      </c>
+      <c r="H14" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I14" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J14" t="str">
+        <v>PAÑO LUSTRE PICO ROJO</v>
+      </c>
+      <c r="K14" t="str">
+        <v>P0001</v>
+      </c>
+      <c r="L14" s="1">
+        <v>4</v>
+      </c>
+      <c r="M14" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N14" s="2">
+        <v>8858</v>
+      </c>
+      <c r="O14" s="2">
+        <v>35432</v>
+      </c>
+      <c r="P14" t="str">
+        <v>Solicitud N° 197</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B15" t="str">
+        <v>09:00 a. m.</v>
+      </c>
+      <c r="C15" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D15" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Ruiz Ernan Eleuterio</v>
+      </c>
+      <c r="F15" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G15" t="str">
+        <v>55-3</v>
+      </c>
+      <c r="H15" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I15" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J15" t="str">
+        <v>LIJA AL AGUA AA #600</v>
+      </c>
+      <c r="K15" t="str">
+        <v>L0019</v>
+      </c>
+      <c r="L15" s="1">
+        <v>10</v>
+      </c>
+      <c r="M15" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N15" s="2">
+        <v>580.7774</v>
+      </c>
+      <c r="O15" s="2">
+        <v>5807.77</v>
+      </c>
+      <c r="P15" t="str">
+        <v>Solicitud N° 197</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B16" t="str">
+        <v>09:00 a. m.</v>
+      </c>
+      <c r="C16" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D16" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Ruiz Ernan Eleuterio</v>
+      </c>
+      <c r="F16" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G16" t="str">
+        <v>55-3</v>
+      </c>
+      <c r="H16" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I16" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J16" t="str">
+        <v>LIJA A/AGUA AA MICROGRANO#1200</v>
+      </c>
+      <c r="K16" t="str">
+        <v>L0021</v>
+      </c>
+      <c r="L16" s="1">
+        <v>10</v>
+      </c>
+      <c r="M16" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N16" s="2">
+        <v>905.8421</v>
+      </c>
+      <c r="O16" s="2">
+        <v>9058.42</v>
+      </c>
+      <c r="P16" t="str">
+        <v>Solicitud N° 197</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B17" t="str">
+        <v>09:00 a. m.</v>
+      </c>
+      <c r="C17" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D17" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Ruiz Ernan Eleuterio</v>
+      </c>
+      <c r="F17" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G17" t="str">
+        <v>55-3</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I17" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J17" t="str">
+        <v>LIJA IMPORTADA NO PAST #400</v>
+      </c>
+      <c r="K17" t="str">
+        <v>L0072</v>
+      </c>
+      <c r="L17" s="1">
+        <v>5</v>
+      </c>
+      <c r="M17" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N17" s="2">
+        <v>539</v>
+      </c>
+      <c r="O17" s="2">
+        <v>2695</v>
+      </c>
+      <c r="P17" t="str">
+        <v>Solicitud N° 197</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B18" t="str">
+        <v>09:43 a. m.</v>
+      </c>
+      <c r="C18" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D18" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Curatitoli Damian</v>
+      </c>
+      <c r="F18" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G18" t="str">
+        <v>55-2</v>
+      </c>
+      <c r="H18" t="str">
+        <v/>
+      </c>
+      <c r="I18" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J18" t="str">
+        <v>PAÑO LUSTRE PICO ROJO</v>
+      </c>
+      <c r="K18" t="str">
+        <v>P0001</v>
+      </c>
+      <c r="L18" s="1">
+        <v>1</v>
+      </c>
+      <c r="M18" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N18" s="2">
+        <v>8858</v>
+      </c>
+      <c r="O18" s="2">
+        <v>8858</v>
+      </c>
+      <c r="P18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B19" t="str">
+        <v>09:51 a. m.</v>
+      </c>
+      <c r="C19" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D19" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Suarez Roberto Sebastian</v>
+      </c>
+      <c r="F19" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+      <c r="H19" t="str">
+        <v>Carpintería</v>
+      </c>
+      <c r="I19" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J19" t="str">
+        <v>Disco de Lija 115mm #60</v>
+      </c>
+      <c r="K19" t="str">
+        <v>D0007</v>
+      </c>
+      <c r="L19" s="1">
+        <v>1</v>
+      </c>
+      <c r="M19" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N19" s="2">
+        <v>1324.4</v>
+      </c>
+      <c r="O19" s="2">
+        <v>1324.4</v>
+      </c>
+      <c r="P19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B20" t="str">
+        <v>09:51 a. m.</v>
+      </c>
+      <c r="C20" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D20" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Suarez Roberto Sebastian</v>
+      </c>
+      <c r="F20" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
+      <c r="H20" t="str">
+        <v>Carpintería</v>
+      </c>
+      <c r="I20" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J20" t="str">
+        <v>MAMELUCO BLANCO LAMINADO</v>
+      </c>
+      <c r="K20" t="str">
+        <v>M0001</v>
+      </c>
+      <c r="L20" s="1">
+        <v>1</v>
+      </c>
+      <c r="M20" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N20" s="2">
+        <v>5143.0949</v>
+      </c>
+      <c r="O20" s="2">
+        <v>5143.09</v>
+      </c>
+      <c r="P20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B21" t="str">
+        <v>09:51 a. m.</v>
+      </c>
+      <c r="C21" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D21" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Suarez Roberto Sebastian</v>
+      </c>
+      <c r="F21" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+      <c r="H21" t="str">
+        <v>Carpintería</v>
+      </c>
+      <c r="I21" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J21" t="str">
+        <v>Disco de Lija 115mm #36</v>
+      </c>
+      <c r="K21" t="str">
+        <v>D0005</v>
+      </c>
+      <c r="L21" s="1">
+        <v>1</v>
+      </c>
+      <c r="M21" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N21" s="2">
+        <v>1524.6</v>
+      </c>
+      <c r="O21" s="2">
+        <v>1524.6</v>
+      </c>
+      <c r="P21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B22" t="str">
+        <v>09:52 a. m.</v>
+      </c>
+      <c r="C22" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D22" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Indaburu Daniel Norberto</v>
+      </c>
+      <c r="F22" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G22" t="str">
+        <v>55-1</v>
+      </c>
+      <c r="H22" t="str">
+        <v/>
+      </c>
+      <c r="I22" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J22" t="str">
+        <v>MECHA DIAM 3,25</v>
+      </c>
+      <c r="K22" t="str">
+        <v>M0028</v>
+      </c>
+      <c r="L22" s="1">
+        <v>1</v>
+      </c>
+      <c r="M22" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N22" s="2">
+        <v>995.26</v>
+      </c>
+      <c r="O22" s="2">
+        <v>995.26</v>
+      </c>
+      <c r="P22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B23" t="str">
+        <v>09:52 a. m.</v>
+      </c>
+      <c r="C23" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D23" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Indaburu Daniel Norberto</v>
+      </c>
+      <c r="F23" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G23" t="str">
+        <v>55-1</v>
+      </c>
+      <c r="H23" t="str">
+        <v/>
+      </c>
+      <c r="I23" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J23" t="str">
+        <v>MECHA DIAM 2,50</v>
+      </c>
+      <c r="K23" t="str">
+        <v>M0025</v>
+      </c>
+      <c r="L23" s="1">
+        <v>1</v>
+      </c>
+      <c r="M23" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N23" s="2">
+        <v>803.83</v>
+      </c>
+      <c r="O23" s="2">
+        <v>803.83</v>
+      </c>
+      <c r="P23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B24" t="str">
+        <v>09:52 a. m.</v>
+      </c>
+      <c r="C24" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D24" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Indaburu Daniel Norberto</v>
+      </c>
+      <c r="F24" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G24" t="str">
+        <v>55-1</v>
+      </c>
+      <c r="H24" t="str">
+        <v/>
+      </c>
+      <c r="I24" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J24" t="str">
+        <v>MECHA DIAM 2</v>
+      </c>
+      <c r="K24" t="str">
+        <v>M0023</v>
+      </c>
+      <c r="L24" s="1">
+        <v>1</v>
+      </c>
+      <c r="M24" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N24" s="2">
+        <v>791.68</v>
+      </c>
+      <c r="O24" s="2">
+        <v>791.68</v>
+      </c>
+      <c r="P24" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B25" t="str">
+        <v>09:53 a. m.</v>
+      </c>
+      <c r="C25" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D25" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Curatitoli Damian</v>
+      </c>
+      <c r="F25" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G25" t="str">
+        <v>55-2</v>
+      </c>
+      <c r="H25" t="str">
+        <v/>
+      </c>
+      <c r="I25" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J25" t="str">
+        <v>Sellador 3M PU550 Blanco x 600</v>
+      </c>
+      <c r="K25" t="str">
+        <v>S0003</v>
+      </c>
+      <c r="L25" s="1">
+        <v>3</v>
+      </c>
+      <c r="M25" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N25" s="2">
+        <v>13274.8</v>
+      </c>
+      <c r="O25" s="2">
+        <v>39824.4</v>
+      </c>
+      <c r="P25" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B26" t="str">
+        <v>11:37 a. m.</v>
+      </c>
+      <c r="C26" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D26" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Ruiz Ernan Eleuterio</v>
+      </c>
+      <c r="F26" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G26" t="str">
+        <v>55-4</v>
+      </c>
+      <c r="H26" t="str">
+        <v>Carpintería</v>
+      </c>
+      <c r="I26" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J26" t="str">
+        <v>LIJA IMPORTADA NO PAST #80</v>
+      </c>
+      <c r="K26" t="str">
+        <v>L0062</v>
+      </c>
+      <c r="L26" s="1">
+        <v>7</v>
+      </c>
+      <c r="M26" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N26" s="2">
+        <v>539</v>
+      </c>
+      <c r="O26" s="2">
+        <v>3773</v>
+      </c>
+      <c r="P26" t="str">
+        <v>Solicitud N° 198</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B27" t="str">
+        <v>11:37 a. m.</v>
+      </c>
+      <c r="C27" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D27" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Ruiz Ernan Eleuterio</v>
+      </c>
+      <c r="F27" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G27" t="str">
+        <v>55-4</v>
+      </c>
+      <c r="H27" t="str">
+        <v>Carpintería</v>
+      </c>
+      <c r="I27" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J27" t="str">
+        <v>Masilla Finish Zeocar x 4Kg</v>
+      </c>
+      <c r="K27" t="str">
+        <v>M0015</v>
+      </c>
+      <c r="L27" s="1">
+        <v>1</v>
+      </c>
+      <c r="M27" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N27" s="2">
+        <v>34170</v>
+      </c>
+      <c r="O27" s="2">
+        <v>34170</v>
+      </c>
+      <c r="P27" t="str">
+        <v>Solicitud N° 198</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B28" t="str">
+        <v>11:37 a. m.</v>
+      </c>
+      <c r="C28" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D28" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Ruiz Ernan Eleuterio</v>
+      </c>
+      <c r="F28" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G28" t="str">
+        <v>55-4</v>
+      </c>
+      <c r="H28" t="str">
+        <v>Carpintería</v>
+      </c>
+      <c r="I28" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J28" t="str">
+        <v>Disco orbital 127mm # 60</v>
+      </c>
+      <c r="K28" t="str">
+        <v>D0024</v>
+      </c>
+      <c r="L28" s="1">
+        <v>7</v>
+      </c>
+      <c r="M28" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N28" s="2">
+        <v>310.0059</v>
+      </c>
+      <c r="O28" s="2">
+        <v>2170.04</v>
+      </c>
+      <c r="P28" t="str">
+        <v>Solicitud N° 198</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B29" t="str">
+        <v>11:44 a. m.</v>
+      </c>
+      <c r="C29" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D29" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Lopez Hernan</v>
+      </c>
+      <c r="F29" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G29" t="str">
+        <v>52-25</v>
+      </c>
+      <c r="H29" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I29" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J29" t="str">
+        <v>Cinta papel DobleA VERDE 48mm</v>
+      </c>
+      <c r="K29" t="str">
+        <v>C0032</v>
+      </c>
+      <c r="L29" s="1">
+        <v>2</v>
+      </c>
+      <c r="M29" t="str">
+        <v>rollo</v>
+      </c>
+      <c r="N29" s="2">
+        <v>5287.36</v>
+      </c>
+      <c r="O29" s="2">
+        <v>10574.72</v>
+      </c>
+      <c r="P29" t="str">
+        <v>Solicitud N° 199</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B30" t="str">
+        <v>11:44 a. m.</v>
+      </c>
+      <c r="C30" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D30" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Lopez Hernan</v>
+      </c>
+      <c r="F30" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G30" t="str">
+        <v>52-25</v>
+      </c>
+      <c r="H30" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I30" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J30" t="str">
+        <v>Film x 2400</v>
+      </c>
+      <c r="K30" t="str">
+        <v>F0029</v>
+      </c>
+      <c r="L30" s="1">
+        <v>2</v>
+      </c>
+      <c r="M30" t="str">
+        <v>rollo</v>
+      </c>
+      <c r="N30" s="2">
+        <v>8836.6571</v>
+      </c>
+      <c r="O30" s="2">
+        <v>17673.31</v>
+      </c>
+      <c r="P30" t="str">
+        <v>Solicitud N° 199</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B31" t="str">
+        <v>11:44 a. m.</v>
+      </c>
+      <c r="C31" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D31" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Lopez Hernan</v>
+      </c>
+      <c r="F31" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G31" t="str">
+        <v>52-25</v>
+      </c>
+      <c r="H31" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I31" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J31" t="str">
+        <v>Cinta papel DobleA VERDE 18mm</v>
+      </c>
+      <c r="K31" t="str">
+        <v>C0031</v>
+      </c>
+      <c r="L31" s="1">
+        <v>2</v>
+      </c>
+      <c r="M31" t="str">
+        <v>rollo</v>
+      </c>
+      <c r="N31" s="2">
+        <v>2038.4</v>
+      </c>
+      <c r="O31" s="2">
+        <v>4076.8</v>
+      </c>
+      <c r="P31" t="str">
+        <v>Solicitud N° 199</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B32" t="str">
+        <v>11:44 a. m.</v>
+      </c>
+      <c r="C32" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D32" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Lopez Hernan</v>
+      </c>
+      <c r="F32" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G32" t="str">
+        <v>52-25</v>
+      </c>
+      <c r="H32" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I32" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J32" t="str">
+        <v>Trapo Blanco CAMISETA x Kilo</v>
+      </c>
+      <c r="K32" t="str">
+        <v>T0009</v>
+      </c>
+      <c r="L32" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="M32" t="str">
+        <v>kg</v>
+      </c>
+      <c r="N32" s="2">
+        <v>3280</v>
+      </c>
+      <c r="O32" s="2">
+        <v>1640</v>
+      </c>
+      <c r="P32" t="str">
+        <v>Solicitud N° 199</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B33" t="str">
+        <v>11:44 a. m.</v>
+      </c>
+      <c r="C33" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D33" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Lopez Hernan</v>
+      </c>
+      <c r="F33" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G33" t="str">
+        <v>52-25</v>
+      </c>
+      <c r="H33" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I33" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J33" t="str">
+        <v>PAÑO LUSTRE PICO ROJO</v>
+      </c>
+      <c r="K33" t="str">
+        <v>P0001</v>
+      </c>
+      <c r="L33" s="1">
+        <v>2</v>
+      </c>
+      <c r="M33" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N33" s="2">
+        <v>8858</v>
+      </c>
+      <c r="O33" s="2">
+        <v>17716</v>
+      </c>
+      <c r="P33" t="str">
+        <v>Solicitud N° 199</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B34" t="str">
+        <v>11:44 a. m.</v>
+      </c>
+      <c r="C34" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D34" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Lopez Hernan</v>
+      </c>
+      <c r="F34" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G34" t="str">
+        <v>52-25</v>
+      </c>
+      <c r="H34" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I34" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J34" t="str">
+        <v>LIJA EN BANDA 6300 X 150 #40</v>
+      </c>
+      <c r="K34" t="str">
+        <v>L0028</v>
+      </c>
+      <c r="L34" s="1">
+        <v>3</v>
+      </c>
+      <c r="M34" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N34" s="2">
+        <v>27657.6329</v>
+      </c>
+      <c r="O34" s="2">
+        <v>82972.9</v>
+      </c>
+      <c r="P34" t="str">
+        <v>Solicitud N° 199</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B35" t="str">
+        <v>11:44 a. m.</v>
+      </c>
+      <c r="C35" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D35" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Lopez Hernan</v>
+      </c>
+      <c r="F35" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G35" t="str">
+        <v>52-25</v>
+      </c>
+      <c r="H35" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I35" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J35" t="str">
+        <v>Estopa Blanca Lustre- x Kg</v>
+      </c>
+      <c r="K35" t="str">
+        <v>E0011</v>
+      </c>
+      <c r="L35" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="M35" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N35" s="2">
+        <v>2380</v>
+      </c>
+      <c r="O35" s="2">
+        <v>1190</v>
+      </c>
+      <c r="P35" t="str">
+        <v>Solicitud N° 199</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B36" t="str">
+        <v>11:44 a. m.</v>
+      </c>
+      <c r="C36" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D36" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Lopez Hernan</v>
+      </c>
+      <c r="F36" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G36" t="str">
+        <v>52-25</v>
+      </c>
+      <c r="H36" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I36" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J36" t="str">
+        <v>LIJA EN BANDA 6300 X 150 #60</v>
+      </c>
+      <c r="K36" t="str">
+        <v>L0029</v>
+      </c>
+      <c r="L36" s="1">
+        <v>3</v>
+      </c>
+      <c r="M36" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N36" s="2">
+        <v>23245.5541</v>
+      </c>
+      <c r="O36" s="2">
+        <v>69736.66</v>
+      </c>
+      <c r="P36" t="str">
+        <v>Solicitud N° 199</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B37" t="str">
+        <v>11:44 a. m.</v>
+      </c>
+      <c r="C37" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D37" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Lopez Hernan</v>
+      </c>
+      <c r="F37" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G37" t="str">
+        <v>52-25</v>
+      </c>
+      <c r="H37" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I37" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J37" t="str">
+        <v>Masilla Zeocar Azul x 1Kg</v>
+      </c>
+      <c r="K37" t="str">
+        <v>M0016</v>
+      </c>
+      <c r="L37" s="1">
+        <v>1</v>
+      </c>
+      <c r="M37" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N37" s="2">
+        <v>10998.0455</v>
+      </c>
+      <c r="O37" s="2">
+        <v>10998.05</v>
+      </c>
+      <c r="P37" t="str">
+        <v>Solicitud N° 199</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B38" t="str">
+        <v>11:47 a. m.</v>
+      </c>
+      <c r="C38" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D38" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E38" t="str">
+        <v>VILLAFAÑE</v>
+      </c>
+      <c r="F38" t="str">
+        <v>manual</v>
+      </c>
+      <c r="G38" t="str">
+        <v>55-1</v>
+      </c>
+      <c r="H38" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I38" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J38" t="str">
+        <v>Cinta papel DobleA VERDE 48mm</v>
+      </c>
+      <c r="K38" t="str">
+        <v>C0032</v>
+      </c>
+      <c r="L38" s="1">
+        <v>2</v>
+      </c>
+      <c r="M38" t="str">
+        <v>rollo</v>
+      </c>
+      <c r="N38" s="2">
+        <v>5287.36</v>
+      </c>
+      <c r="O38" s="2">
+        <v>10574.72</v>
+      </c>
+      <c r="P38" t="str">
+        <v>Solicitud N° 200</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B39" t="str">
+        <v>11:47 a. m.</v>
+      </c>
+      <c r="C39" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D39" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E39" t="str">
+        <v>VILLAFAÑE</v>
+      </c>
+      <c r="F39" t="str">
+        <v>manual</v>
+      </c>
+      <c r="G39" t="str">
+        <v>55-1</v>
+      </c>
+      <c r="H39" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I39" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J39" t="str">
+        <v>Pasta Fina Zeocar X 1kg</v>
+      </c>
+      <c r="K39" t="str">
+        <v>P0005</v>
+      </c>
+      <c r="L39" s="1">
+        <v>1</v>
+      </c>
+      <c r="M39" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N39" s="2">
+        <v>12220</v>
+      </c>
+      <c r="O39" s="2">
+        <v>12220</v>
+      </c>
+      <c r="P39" t="str">
+        <v>Solicitud N° 200</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B40" t="str">
+        <v>11:47 a. m.</v>
+      </c>
+      <c r="C40" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D40" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E40" t="str">
+        <v>VILLAFAÑE</v>
+      </c>
+      <c r="F40" t="str">
+        <v>manual</v>
+      </c>
+      <c r="G40" t="str">
+        <v>55-1</v>
+      </c>
+      <c r="H40" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I40" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J40" t="str">
+        <v>Cinta papel DobleA VERDE 18mm</v>
+      </c>
+      <c r="K40" t="str">
+        <v>C0031</v>
+      </c>
+      <c r="L40" s="1">
+        <v>2</v>
+      </c>
+      <c r="M40" t="str">
+        <v>rollo</v>
+      </c>
+      <c r="N40" s="2">
+        <v>2038.4</v>
+      </c>
+      <c r="O40" s="2">
+        <v>4076.8</v>
+      </c>
+      <c r="P40" t="str">
+        <v>Solicitud N° 200</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B41" t="str">
+        <v>11:47 a. m.</v>
+      </c>
+      <c r="C41" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D41" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E41" t="str">
+        <v>VILLAFAÑE</v>
+      </c>
+      <c r="F41" t="str">
+        <v>manual</v>
+      </c>
+      <c r="G41" t="str">
+        <v>55-1</v>
+      </c>
+      <c r="H41" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I41" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J41" t="str">
+        <v>PAÑO LUSTRE PICO ROJO</v>
+      </c>
+      <c r="K41" t="str">
+        <v>P0001</v>
+      </c>
+      <c r="L41" s="1">
+        <v>4</v>
+      </c>
+      <c r="M41" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N41" s="2">
+        <v>8858</v>
+      </c>
+      <c r="O41" s="2">
+        <v>35432</v>
+      </c>
+      <c r="P41" t="str">
+        <v>Solicitud N° 200</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B42" t="str">
+        <v>11:47 a. m.</v>
+      </c>
+      <c r="C42" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D42" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E42" t="str">
+        <v>VILLAFAÑE</v>
+      </c>
+      <c r="F42" t="str">
+        <v>manual</v>
+      </c>
+      <c r="G42" t="str">
+        <v>55-1</v>
+      </c>
+      <c r="H42" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I42" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J42" t="str">
+        <v>Estopa Blanca Lustre- x Kg</v>
+      </c>
+      <c r="K42" t="str">
+        <v>E0011</v>
+      </c>
+      <c r="L42" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="M42" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N42" s="2">
+        <v>2380</v>
+      </c>
+      <c r="O42" s="2">
+        <v>1190</v>
+      </c>
+      <c r="P42" t="str">
+        <v>Solicitud N° 200</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B43" t="str">
+        <v>11:47 a. m.</v>
+      </c>
+      <c r="C43" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D43" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E43" t="str">
+        <v>VILLAFAÑE</v>
+      </c>
+      <c r="F43" t="str">
+        <v>manual</v>
+      </c>
+      <c r="G43" t="str">
+        <v>55-1</v>
+      </c>
+      <c r="H43" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I43" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J43" t="str">
+        <v>LIJA A/AGUA AA MICROGRANO#1200</v>
+      </c>
+      <c r="K43" t="str">
+        <v>L0021</v>
+      </c>
+      <c r="L43" s="1">
+        <v>10</v>
+      </c>
+      <c r="M43" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N43" s="2">
+        <v>905.8421</v>
+      </c>
+      <c r="O43" s="2">
+        <v>9058.42</v>
+      </c>
+      <c r="P43" t="str">
+        <v>Solicitud N° 200</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B44" t="str">
+        <v>11:47 a. m.</v>
+      </c>
+      <c r="C44" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D44" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E44" t="str">
+        <v>VILLAFAÑE</v>
+      </c>
+      <c r="F44" t="str">
+        <v>manual</v>
+      </c>
+      <c r="G44" t="str">
+        <v>55-1</v>
+      </c>
+      <c r="H44" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I44" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J44" t="str">
+        <v>LIJA IMPORTADA NO PAST #400</v>
+      </c>
+      <c r="K44" t="str">
+        <v>L0072</v>
+      </c>
+      <c r="L44" s="1">
+        <v>10</v>
+      </c>
+      <c r="M44" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N44" s="2">
+        <v>539</v>
+      </c>
+      <c r="O44" s="2">
+        <v>5390</v>
+      </c>
+      <c r="P44" t="str">
+        <v>Solicitud N° 200</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B45" t="str">
+        <v>11:49 a. m.</v>
+      </c>
+      <c r="C45" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D45" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Robledo Pablo Sebastian</v>
+      </c>
+      <c r="F45" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G45" t="str">
+        <v/>
+      </c>
+      <c r="H45" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I45" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J45" t="str">
+        <v>LIJA IMPORTADA NO PAST #80</v>
+      </c>
+      <c r="K45" t="str">
+        <v>L0062</v>
+      </c>
+      <c r="L45" s="1">
+        <v>15</v>
+      </c>
+      <c r="M45" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N45" s="2">
+        <v>539</v>
+      </c>
+      <c r="O45" s="2">
+        <v>8085</v>
+      </c>
+      <c r="P45" t="str">
+        <v>Solicitud N° 201</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B46" t="str">
+        <v>11:49 a. m.</v>
+      </c>
+      <c r="C46" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D46" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E46" t="str">
+        <v>Robledo Pablo Sebastian</v>
+      </c>
+      <c r="F46" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G46" t="str">
+        <v/>
+      </c>
+      <c r="H46" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I46" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J46" t="str">
+        <v>Masilla Finish Zeocar x 4Kg</v>
+      </c>
+      <c r="K46" t="str">
+        <v>M0015</v>
+      </c>
+      <c r="L46" s="1">
+        <v>1</v>
+      </c>
+      <c r="M46" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N46" s="2">
+        <v>34170</v>
+      </c>
+      <c r="O46" s="2">
+        <v>34170</v>
+      </c>
+      <c r="P46" t="str">
+        <v>Solicitud N° 201</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B47" t="str">
+        <v>11:49 a. m.</v>
+      </c>
+      <c r="C47" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D47" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E47" t="str">
+        <v>Robledo Pablo Sebastian</v>
+      </c>
+      <c r="F47" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G47" t="str">
+        <v/>
+      </c>
+      <c r="H47" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I47" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J47" t="str">
+        <v>LIJA IMPORTADA NO PAST #150</v>
+      </c>
+      <c r="K47" t="str">
+        <v>L0065</v>
+      </c>
+      <c r="L47" s="1">
+        <v>15</v>
+      </c>
+      <c r="M47" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N47" s="2">
+        <v>539</v>
+      </c>
+      <c r="O47" s="2">
+        <v>8085</v>
+      </c>
+      <c r="P47" t="str">
+        <v>Solicitud N° 201</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B48" t="str">
+        <v>11:49 a. m.</v>
+      </c>
+      <c r="C48" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D48" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E48" t="str">
+        <v>Robledo Pablo Sebastian</v>
+      </c>
+      <c r="F48" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G48" t="str">
+        <v/>
+      </c>
+      <c r="H48" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I48" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J48" t="str">
+        <v>LIJA A/AGUA AA MICROGRANO#2000</v>
+      </c>
+      <c r="K48" t="str">
+        <v>L0023</v>
+      </c>
+      <c r="L48" s="1">
+        <v>20</v>
+      </c>
+      <c r="M48" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N48" s="2">
+        <v>1334.9292</v>
+      </c>
+      <c r="O48" s="2">
+        <v>26698.58</v>
+      </c>
+      <c r="P48" t="str">
+        <v>Solicitud N° 201</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B49" t="str">
+        <v>11:49 a. m.</v>
+      </c>
+      <c r="C49" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D49" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E49" t="str">
+        <v>Robledo Pablo Sebastian</v>
+      </c>
+      <c r="F49" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G49" t="str">
+        <v/>
+      </c>
+      <c r="H49" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I49" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J49" t="str">
+        <v>PAÑO LUSTRE PICO ROJO</v>
+      </c>
+      <c r="K49" t="str">
+        <v>P0001</v>
+      </c>
+      <c r="L49" s="1">
+        <v>6</v>
+      </c>
+      <c r="M49" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N49" s="2">
+        <v>8858</v>
+      </c>
+      <c r="O49" s="2">
+        <v>53148</v>
+      </c>
+      <c r="P49" t="str">
+        <v>Solicitud N° 201</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B50" t="str">
+        <v>11:49 a. m.</v>
+      </c>
+      <c r="C50" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D50" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E50" t="str">
+        <v>Robledo Pablo Sebastian</v>
+      </c>
+      <c r="F50" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G50" t="str">
+        <v/>
+      </c>
+      <c r="H50" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I50" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J50" t="str">
+        <v>Pincel Nº 20 - Cerda CHINA</v>
+      </c>
+      <c r="K50" t="str">
+        <v>P0017</v>
+      </c>
+      <c r="L50" s="1">
+        <v>5</v>
+      </c>
+      <c r="M50" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N50" s="2">
+        <v>832</v>
+      </c>
+      <c r="O50" s="2">
+        <v>4160</v>
+      </c>
+      <c r="P50" t="str">
+        <v>Solicitud N° 201</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B51" t="str">
+        <v>11:49 a. m.</v>
+      </c>
+      <c r="C51" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D51" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E51" t="str">
+        <v>Robledo Pablo Sebastian</v>
+      </c>
+      <c r="F51" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G51" t="str">
+        <v/>
+      </c>
+      <c r="H51" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I51" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J51" t="str">
+        <v>LIJA AL AGUA AA #600</v>
+      </c>
+      <c r="K51" t="str">
+        <v>L0019</v>
+      </c>
+      <c r="L51" s="1">
+        <v>20</v>
+      </c>
+      <c r="M51" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N51" s="2">
+        <v>580.7774</v>
+      </c>
+      <c r="O51" s="2">
+        <v>11615.55</v>
+      </c>
+      <c r="P51" t="str">
+        <v>Solicitud N° 201</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B52" t="str">
+        <v>11:49 a. m.</v>
+      </c>
+      <c r="C52" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D52" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E52" t="str">
+        <v>Robledo Pablo Sebastian</v>
+      </c>
+      <c r="F52" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G52" t="str">
+        <v/>
+      </c>
+      <c r="H52" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I52" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J52" t="str">
+        <v>LIJA A/AGUA AA MICROGRANO#1000</v>
+      </c>
+      <c r="K52" t="str">
+        <v>L0020</v>
+      </c>
+      <c r="L52" s="1">
+        <v>20</v>
+      </c>
+      <c r="M52" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N52" s="2">
+        <v>905.8421</v>
+      </c>
+      <c r="O52" s="2">
+        <v>18116.84</v>
+      </c>
+      <c r="P52" t="str">
+        <v>Solicitud N° 201</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B53" t="str">
+        <v>11:49 a. m.</v>
+      </c>
+      <c r="C53" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D53" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E53" t="str">
+        <v>Robledo Pablo Sebastian</v>
+      </c>
+      <c r="F53" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G53" t="str">
+        <v/>
+      </c>
+      <c r="H53" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I53" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J53" t="str">
+        <v>Masilla Zeocar Azul x 1Kg</v>
+      </c>
+      <c r="K53" t="str">
+        <v>M0016</v>
+      </c>
+      <c r="L53" s="1">
+        <v>1</v>
+      </c>
+      <c r="M53" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N53" s="2">
+        <v>10998.0455</v>
+      </c>
+      <c r="O53" s="2">
+        <v>10998.05</v>
+      </c>
+      <c r="P53" t="str">
+        <v>Solicitud N° 201</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B54" t="str">
+        <v>11:49 a. m.</v>
+      </c>
+      <c r="C54" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D54" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E54" t="str">
+        <v>Robledo Pablo Sebastian</v>
+      </c>
+      <c r="F54" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G54" t="str">
+        <v/>
+      </c>
+      <c r="H54" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I54" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J54" t="str">
+        <v>DILUYENTE x Lt</v>
+      </c>
+      <c r="K54" t="str">
+        <v>D000111</v>
+      </c>
+      <c r="L54" s="1">
+        <v>1</v>
+      </c>
+      <c r="M54" t="str">
+        <v>litro</v>
+      </c>
+      <c r="N54" s="2">
+        <v>3341.8</v>
+      </c>
+      <c r="O54" s="2">
+        <v>3341.8</v>
+      </c>
+      <c r="P54" t="str">
+        <v>Solicitud N° 201</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B55" t="str">
+        <v>12:37 p. m.</v>
+      </c>
+      <c r="C55" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D55" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E55" t="str">
+        <v>Robledo Pablo Sebastian</v>
+      </c>
+      <c r="F55" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G55" t="str">
+        <v/>
+      </c>
+      <c r="H55" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I55" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J55" t="str">
+        <v>Pasta Fina Zeocar X 1kg</v>
+      </c>
+      <c r="K55" t="str">
+        <v>P0005</v>
+      </c>
+      <c r="L55" s="1">
+        <v>2</v>
+      </c>
+      <c r="M55" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N55" s="2">
+        <v>12220</v>
+      </c>
+      <c r="O55" s="2">
+        <v>24440</v>
+      </c>
+      <c r="P55" t="str">
+        <v>Solicitud N° 202</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B56" t="str">
+        <v>12:37 p. m.</v>
+      </c>
+      <c r="C56" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D56" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E56" t="str">
+        <v>Robledo Pablo Sebastian</v>
+      </c>
+      <c r="F56" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G56" t="str">
+        <v/>
+      </c>
+      <c r="H56" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I56" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J56" t="str">
+        <v>FILTRO PINTURA x10uni</v>
+      </c>
+      <c r="K56" t="str">
+        <v>F00371</v>
+      </c>
+      <c r="L56" s="1">
+        <v>1</v>
+      </c>
+      <c r="M56" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N56" s="2">
+        <v>214.988</v>
+      </c>
+      <c r="O56" s="2">
+        <v>214.99</v>
+      </c>
+      <c r="P56" t="str">
+        <v>Solicitud N° 202</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B57" t="str">
+        <v>12:37 p. m.</v>
+      </c>
+      <c r="C57" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D57" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E57" t="str">
+        <v>Robledo Pablo Sebastian</v>
+      </c>
+      <c r="F57" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G57" t="str">
+        <v/>
+      </c>
+      <c r="H57" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I57" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J57" t="str">
+        <v>Disco orbital 127mm # 100</v>
+      </c>
+      <c r="K57" t="str">
+        <v>D0026</v>
+      </c>
+      <c r="L57" s="1">
+        <v>15</v>
+      </c>
+      <c r="M57" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N57" s="2">
+        <v>207.7008</v>
+      </c>
+      <c r="O57" s="2">
+        <v>3115.51</v>
+      </c>
+      <c r="P57" t="str">
+        <v>Solicitud N° 202</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B58" t="str">
+        <v>12:37 p. m.</v>
+      </c>
+      <c r="C58" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D58" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E58" t="str">
+        <v>Robledo Pablo Sebastian</v>
+      </c>
+      <c r="F58" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G58" t="str">
+        <v/>
+      </c>
+      <c r="H58" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I58" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J58" t="str">
+        <v>LIJA IMPORTADA NO PAST #150</v>
+      </c>
+      <c r="K58" t="str">
+        <v>L0065</v>
+      </c>
+      <c r="L58" s="1">
+        <v>15</v>
+      </c>
+      <c r="M58" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N58" s="2">
+        <v>539</v>
+      </c>
+      <c r="O58" s="2">
+        <v>8085</v>
+      </c>
+      <c r="P58" t="str">
+        <v>Solicitud N° 202</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B59" t="str">
+        <v>12:37 p. m.</v>
+      </c>
+      <c r="C59" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D59" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E59" t="str">
+        <v>Robledo Pablo Sebastian</v>
+      </c>
+      <c r="F59" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G59" t="str">
+        <v/>
+      </c>
+      <c r="H59" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I59" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J59" t="str">
+        <v>LIJA AL AGUA AA #400</v>
+      </c>
+      <c r="K59" t="str">
+        <v>L0018</v>
+      </c>
+      <c r="L59" s="1">
+        <v>20</v>
+      </c>
+      <c r="M59" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N59" s="2">
+        <v>580.7774</v>
+      </c>
+      <c r="O59" s="2">
+        <v>11615.55</v>
+      </c>
+      <c r="P59" t="str">
+        <v>Solicitud N° 202</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B60" t="str">
+        <v>12:37 p. m.</v>
+      </c>
+      <c r="C60" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D60" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E60" t="str">
+        <v>Robledo Pablo Sebastian</v>
+      </c>
+      <c r="F60" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G60" t="str">
+        <v/>
+      </c>
+      <c r="H60" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I60" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J60" t="str">
+        <v>PAÑO LUSTRE PICO ROJO</v>
+      </c>
+      <c r="K60" t="str">
+        <v>P0001</v>
+      </c>
+      <c r="L60" s="1">
+        <v>6</v>
+      </c>
+      <c r="M60" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N60" s="2">
+        <v>8858</v>
+      </c>
+      <c r="O60" s="2">
+        <v>53148</v>
+      </c>
+      <c r="P60" t="str">
+        <v>Solicitud N° 202</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B61" t="str">
+        <v>12:37 p. m.</v>
+      </c>
+      <c r="C61" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D61" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E61" t="str">
+        <v>Robledo Pablo Sebastian</v>
+      </c>
+      <c r="F61" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G61" t="str">
+        <v/>
+      </c>
+      <c r="H61" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I61" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J61" t="str">
+        <v>LIJA AL AGUA AA #600</v>
+      </c>
+      <c r="K61" t="str">
+        <v>L0019</v>
+      </c>
+      <c r="L61" s="1">
+        <v>20</v>
+      </c>
+      <c r="M61" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N61" s="2">
+        <v>580.7774</v>
+      </c>
+      <c r="O61" s="2">
+        <v>11615.55</v>
+      </c>
+      <c r="P61" t="str">
+        <v>Solicitud N° 202</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B62" t="str">
+        <v>12:37 p. m.</v>
+      </c>
+      <c r="C62" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D62" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E62" t="str">
+        <v>Robledo Pablo Sebastian</v>
+      </c>
+      <c r="F62" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G62" t="str">
+        <v/>
+      </c>
+      <c r="H62" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I62" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J62" t="str">
+        <v>Estopa Blanca Lustre- x Kg</v>
+      </c>
+      <c r="K62" t="str">
+        <v>E0011</v>
+      </c>
+      <c r="L62" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="M62" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N62" s="2">
+        <v>2380</v>
+      </c>
+      <c r="O62" s="2">
+        <v>1190</v>
+      </c>
+      <c r="P62" t="str">
+        <v>Solicitud N° 202</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B63" t="str">
+        <v>12:37 p. m.</v>
+      </c>
+      <c r="C63" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D63" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E63" t="str">
+        <v>Robledo Pablo Sebastian</v>
+      </c>
+      <c r="F63" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G63" t="str">
+        <v/>
+      </c>
+      <c r="H63" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I63" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J63" t="str">
+        <v>LIJA IMPORTADA NO PAST #220</v>
+      </c>
+      <c r="K63" t="str">
+        <v>L0067</v>
+      </c>
+      <c r="L63" s="1">
+        <v>15</v>
+      </c>
+      <c r="M63" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N63" s="2">
+        <v>539</v>
+      </c>
+      <c r="O63" s="2">
+        <v>8085</v>
+      </c>
+      <c r="P63" t="str">
+        <v>Solicitud N° 202</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B64" t="str">
+        <v>12:37 p. m.</v>
+      </c>
+      <c r="C64" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D64" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E64" t="str">
+        <v>Robledo Pablo Sebastian</v>
+      </c>
+      <c r="F64" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G64" t="str">
+        <v/>
+      </c>
+      <c r="H64" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I64" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J64" t="str">
+        <v>DILUYENTE x Lt</v>
+      </c>
+      <c r="K64" t="str">
+        <v>D000111</v>
+      </c>
+      <c r="L64" s="1">
+        <v>1</v>
+      </c>
+      <c r="M64" t="str">
+        <v>litro</v>
+      </c>
+      <c r="N64" s="2">
+        <v>3341.8</v>
+      </c>
+      <c r="O64" s="2">
+        <v>3341.8</v>
+      </c>
+      <c r="P64" t="str">
+        <v>Solicitud N° 202</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B65" t="str">
+        <v>12:47 p. m.</v>
+      </c>
+      <c r="C65" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D65" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E65" t="str">
+        <v>Frias Luis Ruben</v>
+      </c>
+      <c r="F65" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G65" t="str">
+        <v>43-30</v>
+      </c>
+      <c r="H65" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I65" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J65" t="str">
+        <v>Cinta papel DobleA VERDE 48mm</v>
+      </c>
+      <c r="K65" t="str">
+        <v>C0032</v>
+      </c>
+      <c r="L65" s="1">
+        <v>2</v>
+      </c>
+      <c r="M65" t="str">
+        <v>rollo</v>
+      </c>
+      <c r="N65" s="2">
+        <v>5287.36</v>
+      </c>
+      <c r="O65" s="2">
+        <v>10574.72</v>
+      </c>
+      <c r="P65" t="str">
+        <v>Solicitud N° 203</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B66" t="str">
+        <v>12:47 p. m.</v>
+      </c>
+      <c r="C66" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D66" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E66" t="str">
+        <v>Frias Luis Ruben</v>
+      </c>
+      <c r="F66" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G66" t="str">
+        <v>43-30</v>
+      </c>
+      <c r="H66" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I66" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J66" t="str">
+        <v>Cinta papel DobleA VERDE 18mm</v>
+      </c>
+      <c r="K66" t="str">
+        <v>C0031</v>
+      </c>
+      <c r="L66" s="1">
+        <v>2</v>
+      </c>
+      <c r="M66" t="str">
+        <v>rollo</v>
+      </c>
+      <c r="N66" s="2">
+        <v>2038.4</v>
+      </c>
+      <c r="O66" s="2">
+        <v>4076.8</v>
+      </c>
+      <c r="P66" t="str">
+        <v>Solicitud N° 203</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B67" t="str">
+        <v>12:47 p. m.</v>
+      </c>
+      <c r="C67" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D67" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E67" t="str">
+        <v>Frias Luis Ruben</v>
+      </c>
+      <c r="F67" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G67" t="str">
+        <v>43-30</v>
+      </c>
+      <c r="H67" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I67" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J67" t="str">
+        <v>Trapo Blanco CAMISETA x Kilo</v>
+      </c>
+      <c r="K67" t="str">
+        <v>T0009</v>
+      </c>
+      <c r="L67" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="M67" t="str">
+        <v>kg</v>
+      </c>
+      <c r="N67" s="2">
+        <v>3280</v>
+      </c>
+      <c r="O67" s="2">
+        <v>1640</v>
+      </c>
+      <c r="P67" t="str">
+        <v>Solicitud N° 203</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B68" t="str">
+        <v>12:47 p. m.</v>
+      </c>
+      <c r="C68" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D68" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E68" t="str">
+        <v>Frias Luis Ruben</v>
+      </c>
+      <c r="F68" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G68" t="str">
+        <v>43-30</v>
+      </c>
+      <c r="H68" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I68" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J68" t="str">
+        <v>LIJA EN BANDA 6300 X 150 #40</v>
+      </c>
+      <c r="K68" t="str">
+        <v>L0028</v>
+      </c>
+      <c r="L68" s="1">
+        <v>2</v>
+      </c>
+      <c r="M68" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N68" s="2">
+        <v>27657.6329</v>
+      </c>
+      <c r="O68" s="2">
+        <v>55315.27</v>
+      </c>
+      <c r="P68" t="str">
+        <v>Solicitud N° 203</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B69" t="str">
+        <v>12:47 p. m.</v>
+      </c>
+      <c r="C69" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D69" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E69" t="str">
+        <v>Frias Luis Ruben</v>
+      </c>
+      <c r="F69" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G69" t="str">
+        <v>43-30</v>
+      </c>
+      <c r="H69" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I69" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J69" t="str">
+        <v>Estopa Blanca Lustre- x Kg</v>
+      </c>
+      <c r="K69" t="str">
+        <v>E0011</v>
+      </c>
+      <c r="L69" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="M69" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N69" s="2">
+        <v>2380</v>
+      </c>
+      <c r="O69" s="2">
+        <v>1190</v>
+      </c>
+      <c r="P69" t="str">
+        <v>Solicitud N° 203</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B70" t="str">
+        <v>12:47 p. m.</v>
+      </c>
+      <c r="C70" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D70" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E70" t="str">
+        <v>Frias Luis Ruben</v>
+      </c>
+      <c r="F70" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G70" t="str">
+        <v>43-30</v>
+      </c>
+      <c r="H70" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I70" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J70" t="str">
+        <v>LIJA IMPORTADA NO PAST #100</v>
+      </c>
+      <c r="K70" t="str">
+        <v>L0063</v>
+      </c>
+      <c r="L70" s="1">
+        <v>7</v>
+      </c>
+      <c r="M70" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N70" s="2">
+        <v>539</v>
+      </c>
+      <c r="O70" s="2">
+        <v>3773</v>
+      </c>
+      <c r="P70" t="str">
+        <v>Solicitud N° 203</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B71" t="str">
+        <v>12:47 p. m.</v>
+      </c>
+      <c r="C71" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D71" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E71" t="str">
+        <v>Frias Luis Ruben</v>
+      </c>
+      <c r="F71" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G71" t="str">
+        <v>43-30</v>
+      </c>
+      <c r="H71" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I71" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J71" t="str">
+        <v>LIJA AL AGUA AA #320</v>
+      </c>
+      <c r="K71" t="str">
+        <v>L0016</v>
+      </c>
+      <c r="L71" s="1">
+        <v>7</v>
+      </c>
+      <c r="M71" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N71" s="2">
+        <v>580.7774</v>
+      </c>
+      <c r="O71" s="2">
+        <v>4065.44</v>
+      </c>
+      <c r="P71" t="str">
+        <v>Solicitud N° 203</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B72" t="str">
+        <v>12:47 p. m.</v>
+      </c>
+      <c r="C72" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D72" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E72" t="str">
+        <v>Frias Luis Ruben</v>
+      </c>
+      <c r="F72" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G72" t="str">
+        <v>43-30</v>
+      </c>
+      <c r="H72" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I72" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J72" t="str">
+        <v>LIJA EN BANDA 6300 X 150 #60</v>
+      </c>
+      <c r="K72" t="str">
+        <v>L0029</v>
+      </c>
+      <c r="L72" s="1">
+        <v>2</v>
+      </c>
+      <c r="M72" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N72" s="2">
+        <v>23245.5541</v>
+      </c>
+      <c r="O72" s="2">
+        <v>46491.11</v>
+      </c>
+      <c r="P72" t="str">
+        <v>Solicitud N° 203</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B73" t="str">
+        <v>12:47 p. m.</v>
+      </c>
+      <c r="C73" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D73" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E73" t="str">
+        <v>Frias Luis Ruben</v>
+      </c>
+      <c r="F73" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G73" t="str">
+        <v>43-30</v>
+      </c>
+      <c r="H73" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I73" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J73" t="str">
+        <v>CUTTER ECONOMICO X 18CM</v>
+      </c>
+      <c r="K73" t="str">
+        <v>C0053</v>
+      </c>
+      <c r="L73" s="1">
+        <v>2</v>
+      </c>
+      <c r="M73" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N73" s="2">
+        <v>1596</v>
+      </c>
+      <c r="O73" s="2">
+        <v>3192</v>
+      </c>
+      <c r="P73" t="str">
+        <v>Solicitud N° 203</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B74" t="str">
+        <v>12:47 p. m.</v>
+      </c>
+      <c r="C74" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D74" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E74" t="str">
+        <v>Frias Luis Ruben</v>
+      </c>
+      <c r="F74" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G74" t="str">
+        <v>43-30</v>
+      </c>
+      <c r="H74" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I74" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J74" t="str">
+        <v>LIJA A/AGUA AA MICROGRANO#1000</v>
+      </c>
+      <c r="K74" t="str">
+        <v>L0020</v>
+      </c>
+      <c r="L74" s="1">
+        <v>7</v>
+      </c>
+      <c r="M74" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N74" s="2">
+        <v>905.8421</v>
+      </c>
+      <c r="O74" s="2">
+        <v>6340.89</v>
+      </c>
+      <c r="P74" t="str">
+        <v>Solicitud N° 203</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B75" t="str">
+        <v>12:47 p. m.</v>
+      </c>
+      <c r="C75" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D75" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E75" t="str">
+        <v>Frias Luis Ruben</v>
+      </c>
+      <c r="F75" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G75" t="str">
+        <v>43-30</v>
+      </c>
+      <c r="H75" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I75" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J75" t="str">
+        <v>LIJA IMPORTADA NO PAST #400</v>
+      </c>
+      <c r="K75" t="str">
+        <v>L0072</v>
+      </c>
+      <c r="L75" s="1">
+        <v>7</v>
+      </c>
+      <c r="M75" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N75" s="2">
+        <v>539</v>
+      </c>
+      <c r="O75" s="2">
+        <v>3773</v>
+      </c>
+      <c r="P75" t="str">
+        <v>Solicitud N° 203</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B76" t="str">
+        <v>12:47 p. m.</v>
+      </c>
+      <c r="C76" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D76" t="str">
+        <v>planificado</v>
+      </c>
+      <c r="E76" t="str">
+        <v>Frias Luis Ruben</v>
+      </c>
+      <c r="F76" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G76" t="str">
+        <v>43-30</v>
+      </c>
+      <c r="H76" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I76" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J76" t="str">
+        <v>DILUYENTE x Lt</v>
+      </c>
+      <c r="K76" t="str">
+        <v>D000111</v>
+      </c>
+      <c r="L76" s="1">
+        <v>1</v>
+      </c>
+      <c r="M76" t="str">
+        <v>litro</v>
+      </c>
+      <c r="N76" s="2">
+        <v>3341.8</v>
+      </c>
+      <c r="O76" s="2">
+        <v>3341.8</v>
+      </c>
+      <c r="P76" t="str">
+        <v>Solicitud N° 203</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B77" t="str">
+        <v>12:49 p. m.</v>
+      </c>
+      <c r="C77" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D77" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E77" t="str">
+        <v>Frias Luis Ruben</v>
+      </c>
+      <c r="F77" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G77" t="str">
+        <v/>
+      </c>
+      <c r="H77" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I77" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J77" t="str">
+        <v>Disco orbital 127mm # 60</v>
+      </c>
+      <c r="K77" t="str">
+        <v>D0024</v>
+      </c>
+      <c r="L77" s="1">
+        <v>2</v>
+      </c>
+      <c r="M77" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N77" s="2">
+        <v>310.0059</v>
+      </c>
+      <c r="O77" s="2">
+        <v>620.01</v>
+      </c>
+      <c r="P77" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B78" t="str">
+        <v>12:49 p. m.</v>
+      </c>
+      <c r="C78" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D78" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E78" t="str">
+        <v>Frias Luis Ruben</v>
+      </c>
+      <c r="F78" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G78" t="str">
+        <v/>
+      </c>
+      <c r="H78" t="str">
+        <v>Pintura</v>
+      </c>
+      <c r="I78" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J78" t="str">
+        <v>Disco orbital 127mm # 80</v>
+      </c>
+      <c r="K78" t="str">
+        <v>D0025</v>
+      </c>
+      <c r="L78" s="1">
+        <v>2</v>
+      </c>
+      <c r="M78" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N78" s="2">
+        <v>310.0059</v>
+      </c>
+      <c r="O78" s="2">
+        <v>620.01</v>
+      </c>
+      <c r="P78" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B79" t="str">
+        <v>01:19 p. m.</v>
+      </c>
+      <c r="C79" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D79" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E79" t="str">
+        <v>Almirón Jonathan Emanuel</v>
+      </c>
+      <c r="F79" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G79" t="str">
+        <v>55-1</v>
+      </c>
+      <c r="H79" t="str">
+        <v/>
+      </c>
+      <c r="I79" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J79" t="str">
+        <v>LIJA AL AGUA AA #400</v>
+      </c>
+      <c r="K79" t="str">
+        <v>L0018</v>
+      </c>
+      <c r="L79" s="1">
+        <v>1</v>
+      </c>
+      <c r="M79" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N79" s="2">
+        <v>580.7774</v>
+      </c>
+      <c r="O79" s="2">
+        <v>580.78</v>
+      </c>
+      <c r="P79" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B80" t="str">
+        <v>01:19 p. m.</v>
+      </c>
+      <c r="C80" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D80" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E80" t="str">
+        <v>Almirón Jonathan Emanuel</v>
+      </c>
+      <c r="F80" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G80" t="str">
+        <v>55-1</v>
+      </c>
+      <c r="H80" t="str">
+        <v/>
+      </c>
+      <c r="I80" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J80" t="str">
+        <v>LIJA AL AGUA AA #600</v>
+      </c>
+      <c r="K80" t="str">
+        <v>L0019</v>
+      </c>
+      <c r="L80" s="1">
+        <v>1</v>
+      </c>
+      <c r="M80" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N80" s="2">
+        <v>580.7774</v>
+      </c>
+      <c r="O80" s="2">
+        <v>580.78</v>
+      </c>
+      <c r="P80" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B81" t="str">
+        <v>01:19 p. m.</v>
+      </c>
+      <c r="C81" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D81" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E81" t="str">
+        <v>Almirón Jonathan Emanuel</v>
+      </c>
+      <c r="F81" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G81" t="str">
+        <v>55-1</v>
+      </c>
+      <c r="H81" t="str">
+        <v/>
+      </c>
+      <c r="I81" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J81" t="str">
+        <v>LIJA A/AGUA AA MICROGRANO#1200</v>
+      </c>
+      <c r="K81" t="str">
+        <v>L0021</v>
+      </c>
+      <c r="L81" s="1">
+        <v>1</v>
+      </c>
+      <c r="M81" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N81" s="2">
+        <v>905.8421</v>
+      </c>
+      <c r="O81" s="2">
+        <v>905.84</v>
+      </c>
+      <c r="P81" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B82" t="str">
+        <v>01:22 p. m.</v>
+      </c>
+      <c r="C82" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D82" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E82" t="str">
+        <v>Salamonini Enzo Ariel</v>
+      </c>
+      <c r="F82" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G82" t="str">
+        <v>37-42</v>
+      </c>
+      <c r="H82" t="str">
+        <v/>
+      </c>
+      <c r="I82" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J82" t="str">
+        <v>POXIPOL 700ml TRANSPARENTE</v>
+      </c>
+      <c r="K82" t="str">
+        <v>P0041TRANS</v>
+      </c>
+      <c r="L82" s="1">
+        <v>1</v>
+      </c>
+      <c r="M82" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N82" s="2">
+        <v>80788.581</v>
+      </c>
+      <c r="O82" s="2">
+        <v>80788.58</v>
+      </c>
+      <c r="P82" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B83" t="str">
+        <v>01:25 p. m.</v>
+      </c>
+      <c r="C83" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D83" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E83" t="str">
+        <v>Ramasanta Gaston</v>
+      </c>
+      <c r="F83" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G83" t="str">
+        <v>55-1</v>
+      </c>
+      <c r="H83" t="str">
+        <v/>
+      </c>
+      <c r="I83" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J83" t="str">
+        <v>MECHA DIAM 2</v>
+      </c>
+      <c r="K83" t="str">
+        <v>M0023</v>
+      </c>
+      <c r="L83" s="1">
+        <v>1</v>
+      </c>
+      <c r="M83" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N83" s="2">
+        <v>791.68</v>
+      </c>
+      <c r="O83" s="2">
+        <v>791.68</v>
+      </c>
+      <c r="P83" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B84" t="str">
+        <v>01:30 p. m.</v>
+      </c>
+      <c r="C84" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D84" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E84" t="str">
+        <v>Salamonini Tomas Angel</v>
+      </c>
+      <c r="F84" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G84" t="str">
+        <v/>
+      </c>
+      <c r="H84" t="str">
+        <v>Otro</v>
+      </c>
+      <c r="I84" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J84" t="str">
+        <v>Fana 96 - Lata x 14 Kg.</v>
+      </c>
+      <c r="K84" t="str">
+        <v>F0022</v>
+      </c>
+      <c r="L84" s="1">
+        <v>1</v>
+      </c>
+      <c r="M84" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N84" s="2">
+        <v>140756</v>
+      </c>
+      <c r="O84" s="2">
+        <v>140756</v>
+      </c>
+      <c r="P84" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B85" t="str">
+        <v>01:38 p. m.</v>
+      </c>
+      <c r="C85" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D85" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E85" t="str">
+        <v>Gavilan Carlos Eloy</v>
+      </c>
+      <c r="F85" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G85" t="str">
+        <v>52-24</v>
+      </c>
+      <c r="H85" t="str">
+        <v/>
+      </c>
+      <c r="I85" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J85" t="str">
+        <v>PUNTAS PH2 X 50MM</v>
+      </c>
+      <c r="K85" t="str">
+        <v>P0055</v>
+      </c>
+      <c r="L85" s="1">
+        <v>1</v>
+      </c>
+      <c r="M85" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N85" s="2">
+        <v>692</v>
+      </c>
+      <c r="O85" s="2">
+        <v>692</v>
+      </c>
+      <c r="P85" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B86" t="str">
+        <v>01:47 p. m.</v>
+      </c>
+      <c r="C86" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D86" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E86" t="str">
+        <v>Sanchez Martin Antonio</v>
+      </c>
+      <c r="F86" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G86" t="str">
+        <v>43-30</v>
+      </c>
+      <c r="H86" t="str">
+        <v/>
+      </c>
+      <c r="I86" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J86" t="str">
+        <v>Disco orbital 127mm # 60</v>
+      </c>
+      <c r="K86" t="str">
+        <v>D0024</v>
+      </c>
+      <c r="L86" s="1">
+        <v>10</v>
+      </c>
+      <c r="M86" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N86" s="2">
+        <v>310.0059</v>
+      </c>
+      <c r="O86" s="2">
+        <v>3100.06</v>
+      </c>
+      <c r="P86" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B87" t="str">
+        <v>01:47 p. m.</v>
+      </c>
+      <c r="C87" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D87" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E87" t="str">
+        <v>Sanchez Martin Antonio</v>
+      </c>
+      <c r="F87" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G87" t="str">
+        <v>43-30</v>
+      </c>
+      <c r="H87" t="str">
+        <v/>
+      </c>
+      <c r="I87" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J87" t="str">
+        <v>Disco orbital 127mm # 80</v>
+      </c>
+      <c r="K87" t="str">
+        <v>D0025</v>
+      </c>
+      <c r="L87" s="1">
+        <v>10</v>
+      </c>
+      <c r="M87" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N87" s="2">
+        <v>310.0059</v>
+      </c>
+      <c r="O87" s="2">
+        <v>3100.06</v>
+      </c>
+      <c r="P87" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B88" t="str">
+        <v>01:55 p. m.</v>
+      </c>
+      <c r="C88" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D88" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E88" t="str">
+        <v>Ramirez Dylan Ezequiel</v>
+      </c>
+      <c r="F88" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G88" t="str">
+        <v>55-1</v>
+      </c>
+      <c r="H88" t="str">
+        <v/>
+      </c>
+      <c r="I88" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J88" t="str">
+        <v>MECHA DIAM 6</v>
+      </c>
+      <c r="K88" t="str">
+        <v>M0039</v>
+      </c>
+      <c r="L88" s="1">
+        <v>2</v>
+      </c>
+      <c r="M88" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N88" s="2">
+        <v>2087.13</v>
+      </c>
+      <c r="O88" s="2">
+        <v>4174.26</v>
+      </c>
+      <c r="P88" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B89" t="str">
+        <v>01:55 p. m.</v>
+      </c>
+      <c r="C89" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D89" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E89" t="str">
+        <v>Ramirez Dylan Ezequiel</v>
+      </c>
+      <c r="F89" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G89" t="str">
+        <v>55-1</v>
+      </c>
+      <c r="H89" t="str">
+        <v/>
+      </c>
+      <c r="I89" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J89" t="str">
+        <v>MECHA DIAM 10</v>
+      </c>
+      <c r="K89" t="str">
+        <v>M0051</v>
+      </c>
+      <c r="L89" s="1">
+        <v>2</v>
+      </c>
+      <c r="M89" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N89" s="2">
+        <v>5254.24</v>
+      </c>
+      <c r="O89" s="2">
+        <v>10508.48</v>
+      </c>
+      <c r="P89" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B90" t="str">
+        <v>01:55 p. m.</v>
+      </c>
+      <c r="C90" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D90" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E90" t="str">
+        <v>Ramirez Dylan Ezequiel</v>
+      </c>
+      <c r="F90" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G90" t="str">
+        <v>55-1</v>
+      </c>
+      <c r="H90" t="str">
+        <v/>
+      </c>
+      <c r="I90" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J90" t="str">
+        <v>MECHA DIAM 7</v>
+      </c>
+      <c r="K90" t="str">
+        <v>M0043</v>
+      </c>
+      <c r="L90" s="1">
+        <v>2</v>
+      </c>
+      <c r="M90" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N90" s="2">
+        <v>2884.15</v>
+      </c>
+      <c r="O90" s="2">
+        <v>5768.3</v>
+      </c>
+      <c r="P90" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B91" t="str">
+        <v>01:55 p. m.</v>
+      </c>
+      <c r="C91" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D91" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E91" t="str">
+        <v>Ramirez Dylan Ezequiel</v>
+      </c>
+      <c r="F91" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G91" t="str">
+        <v>55-1</v>
+      </c>
+      <c r="H91" t="str">
+        <v/>
+      </c>
+      <c r="I91" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J91" t="str">
+        <v>MECHA DIAM 9</v>
+      </c>
+      <c r="K91" t="str">
+        <v>M0049</v>
+      </c>
+      <c r="L91" s="1">
+        <v>2</v>
+      </c>
+      <c r="M91" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N91" s="2">
+        <v>4663.78</v>
+      </c>
+      <c r="O91" s="2">
+        <v>9327.56</v>
+      </c>
+      <c r="P91" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B92" t="str">
+        <v>01:55 p. m.</v>
+      </c>
+      <c r="C92" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D92" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E92" t="str">
+        <v>Ramirez Dylan Ezequiel</v>
+      </c>
+      <c r="F92" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G92" t="str">
+        <v>55-1</v>
+      </c>
+      <c r="H92" t="str">
+        <v/>
+      </c>
+      <c r="I92" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J92" t="str">
+        <v>MECHA DIAM 8</v>
+      </c>
+      <c r="K92" t="str">
+        <v>M0047</v>
+      </c>
+      <c r="L92" s="1">
+        <v>2</v>
+      </c>
+      <c r="M92" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N92" s="2">
+        <v>3619.09</v>
+      </c>
+      <c r="O92" s="2">
+        <v>7238.18</v>
+      </c>
+      <c r="P92" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B93" t="str">
+        <v>02:10 p. m.</v>
+      </c>
+      <c r="C93" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D93" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E93" t="str">
+        <v>Suarez Roberto Sebastian</v>
+      </c>
+      <c r="F93" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G93" t="str">
+        <v>55-4</v>
+      </c>
+      <c r="H93" t="str">
+        <v/>
+      </c>
+      <c r="I93" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J93" t="str">
+        <v>PUNTAS PH1 X 50MM</v>
+      </c>
+      <c r="K93" t="str">
+        <v>P0053</v>
+      </c>
+      <c r="L93" s="1">
+        <v>1</v>
+      </c>
+      <c r="M93" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N93" s="2">
+        <v>692</v>
+      </c>
+      <c r="O93" s="2">
+        <v>692</v>
+      </c>
+      <c r="P93" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B94" t="str">
+        <v>02:29 p. m.</v>
+      </c>
+      <c r="C94" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D94" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E94" t="str">
+        <v>Gomez Matias Facundo</v>
+      </c>
+      <c r="F94" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G94" t="str">
+        <v>52-26</v>
+      </c>
+      <c r="H94" t="str">
+        <v/>
+      </c>
+      <c r="I94" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J94" t="str">
+        <v>Cinta papel DobleA VERDE 48mm</v>
+      </c>
+      <c r="K94" t="str">
+        <v>C0032</v>
+      </c>
+      <c r="L94" s="1">
+        <v>1</v>
+      </c>
+      <c r="M94" t="str">
+        <v>rollo</v>
+      </c>
+      <c r="N94" s="2">
+        <v>5287.36</v>
+      </c>
+      <c r="O94" s="2">
+        <v>5287.36</v>
+      </c>
+      <c r="P94" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B95" t="str">
+        <v>02:29 p. m.</v>
+      </c>
+      <c r="C95" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D95" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E95" t="str">
+        <v>Gomez Matias Facundo</v>
+      </c>
+      <c r="F95" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G95" t="str">
+        <v>52-26</v>
+      </c>
+      <c r="H95" t="str">
+        <v/>
+      </c>
+      <c r="I95" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J95" t="str">
+        <v>Cinta papel DobleA VERDE 18mm</v>
+      </c>
+      <c r="K95" t="str">
+        <v>C0031</v>
+      </c>
+      <c r="L95" s="1">
+        <v>1</v>
+      </c>
+      <c r="M95" t="str">
+        <v>rollo</v>
+      </c>
+      <c r="N95" s="2">
+        <v>2038.4</v>
+      </c>
+      <c r="O95" s="2">
+        <v>2038.4</v>
+      </c>
+      <c r="P95" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B96" t="str">
+        <v>02:31 p. m.</v>
+      </c>
+      <c r="C96" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D96" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E96" t="str">
+        <v>Montesano Tobias Emanuel</v>
+      </c>
+      <c r="F96" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G96" t="str">
+        <v>64-21</v>
+      </c>
+      <c r="H96" t="str">
+        <v/>
+      </c>
+      <c r="I96" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J96" t="str">
+        <v>LIJA EN BANDA 6300 X 150 #60</v>
+      </c>
+      <c r="K96" t="str">
+        <v>L0029</v>
+      </c>
+      <c r="L96" s="1">
+        <v>1</v>
+      </c>
+      <c r="M96" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N96" s="2">
+        <v>23245.5541</v>
+      </c>
+      <c r="O96" s="2">
+        <v>23245.55</v>
+      </c>
+      <c r="P96" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B97" t="str">
+        <v>02:34 p. m.</v>
+      </c>
+      <c r="C97" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D97" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E97" t="str">
+        <v>Gomez Marcos Valentin</v>
+      </c>
+      <c r="F97" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G97" t="str">
+        <v>55-4</v>
+      </c>
+      <c r="H97" t="str">
+        <v/>
+      </c>
+      <c r="I97" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J97" t="str">
+        <v>T118B Hoja calar Blister</v>
+      </c>
+      <c r="K97" t="str">
+        <v>H0010</v>
+      </c>
+      <c r="L97" s="1">
+        <v>2</v>
+      </c>
+      <c r="M97" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N97" s="2">
+        <v>10240.8866</v>
+      </c>
+      <c r="O97" s="2">
+        <v>20481.77</v>
+      </c>
+      <c r="P97" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B98" t="str">
+        <v>02:46 p. m.</v>
+      </c>
+      <c r="C98" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D98" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E98" t="str">
+        <v>Orlando Jeremias David</v>
+      </c>
+      <c r="F98" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G98" t="str">
+        <v>55-4</v>
+      </c>
+      <c r="H98" t="str">
+        <v/>
+      </c>
+      <c r="I98" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J98" t="str">
+        <v>Disco de Lija 180mm #36</v>
+      </c>
+      <c r="K98" t="str">
+        <v>D0013</v>
+      </c>
+      <c r="L98" s="1">
+        <v>2</v>
+      </c>
+      <c r="M98" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N98" s="2">
+        <v>2725.8</v>
+      </c>
+      <c r="O98" s="2">
+        <v>5451.6</v>
+      </c>
+      <c r="P98" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P10"/>
+  <autoFilter ref="A1:P98"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P98"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Consumibles: hojas de blíster sueltas y el Catálogo exige factor al cambiar la unidad
- Las 13 hojas de calar y sierra en blíster se entregan sueltas: unidad hoja,
  compra por blíster de 5 y costo por hoja. Las 2 T118B del 13/10 se
  recargaron como 2 hojas. Migración 20261013190000, ya aplicada.
- Catálogo: no se guarda una unidad de entrega distinta de la de compra (o un
  fraccionado) sin factor; sin él cada metro valía el envase entero (pasó con
  el cartón en rollo). "Revisar unidad" también marca los fraccionados sin
  factor. "hoja" entra en las unidades sugeridas.
- Excel de consumo regenerado: el histórico baja a $12,36 M con las hojas
  valorizadas por hoja.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/entregables/consumibles/consumo-consumibles-2026-10-13.xlsx
+++ b/entregables/consumibles/consumo-consumibles-2026-10-13.xlsx
@@ -23,7 +23,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6">'Por mes y rubro'!$A$1:$D$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7">'Por producto'!$A$1:$H$141</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8">'Sin valorizar'!$A$1:$E$43</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9">'Registro nuevo (desde 13-10)'!$A$1:$P$98</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9">'Registro nuevo (desde 13-10)'!$A$1:$P$101</definedName>
   </definedNames>
 </workbook>
 </file>
@@ -462,7 +462,7 @@
         <v>Valorizado a costo de hoy (pesos sin IVA)</v>
       </c>
       <c r="B7">
-        <v>12597073.93</v>
+        <v>12363996.47</v>
       </c>
     </row>
     <row r="8">
@@ -497,7 +497,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P98"/>
+  <dimension ref="A1:P101"/>
   <cols>
     <col min="1" max="1" width="11.83203125" customWidth="1"/>
     <col min="2" max="2" width="7.83203125" customWidth="1"/>
@@ -5355,16 +5355,16 @@
         <v>2</v>
       </c>
       <c r="M97" t="str">
-        <v>unidad</v>
+        <v>hoja</v>
       </c>
       <c r="N97" s="2">
-        <v>10240.8866</v>
+        <v>2048.1773</v>
       </c>
       <c r="O97" s="2">
-        <v>20481.77</v>
+        <v>4096.35</v>
       </c>
       <c r="P97" t="str">
-        <v/>
+        <v>Recargado en hojas (figuraba como blísteres)</v>
       </c>
     </row>
     <row r="98">
@@ -5417,10 +5417,160 @@
         <v/>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B99" t="str">
+        <v>02:57 p. m.</v>
+      </c>
+      <c r="C99" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D99" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E99" t="str">
+        <v>Piras Pablo Ezequiel</v>
+      </c>
+      <c r="F99" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G99" t="str">
+        <v>55-4</v>
+      </c>
+      <c r="H99" t="str">
+        <v/>
+      </c>
+      <c r="I99" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J99" t="str">
+        <v>Ciano x 25ml</v>
+      </c>
+      <c r="K99" t="str">
+        <v>C0012</v>
+      </c>
+      <c r="L99" s="1">
+        <v>1</v>
+      </c>
+      <c r="M99" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N99" s="2">
+        <v>7571.88</v>
+      </c>
+      <c r="O99" s="2">
+        <v>7571.88</v>
+      </c>
+      <c r="P99" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B100" t="str">
+        <v>03:06 p. m.</v>
+      </c>
+      <c r="C100" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D100" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E100" t="str">
+        <v>Alegre Lucas Emanuel</v>
+      </c>
+      <c r="F100" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G100" t="str">
+        <v>55-3</v>
+      </c>
+      <c r="H100" t="str">
+        <v/>
+      </c>
+      <c r="I100" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J100" t="str">
+        <v>LIJA IMPORTADA NO PAST #80</v>
+      </c>
+      <c r="K100" t="str">
+        <v>L0062</v>
+      </c>
+      <c r="L100" s="1">
+        <v>5</v>
+      </c>
+      <c r="M100" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N100" s="2">
+        <v>539</v>
+      </c>
+      <c r="O100" s="2">
+        <v>2695</v>
+      </c>
+      <c r="P100" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="str">
+        <v>2026-10-13</v>
+      </c>
+      <c r="B101" t="str">
+        <v>03:06 p. m.</v>
+      </c>
+      <c r="C101" t="str">
+        <v>retiro</v>
+      </c>
+      <c r="D101" t="str">
+        <v>mostrador</v>
+      </c>
+      <c r="E101" t="str">
+        <v>Alegre Lucas Emanuel</v>
+      </c>
+      <c r="F101" t="str">
+        <v>sin_tarjeta</v>
+      </c>
+      <c r="G101" t="str">
+        <v>55-3</v>
+      </c>
+      <c r="H101" t="str">
+        <v/>
+      </c>
+      <c r="I101" t="str">
+        <v>Chubut</v>
+      </c>
+      <c r="J101" t="str">
+        <v>LIJA AL AGUA AA #600</v>
+      </c>
+      <c r="K101" t="str">
+        <v>L0019</v>
+      </c>
+      <c r="L101" s="1">
+        <v>1</v>
+      </c>
+      <c r="M101" t="str">
+        <v>unidad</v>
+      </c>
+      <c r="N101" s="2">
+        <v>580.7774</v>
+      </c>
+      <c r="O101" s="2">
+        <v>580.78</v>
+      </c>
+      <c r="P101" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P98"/>
+  <autoFilter ref="A1:P101"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P98"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P101"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8754,16 +8904,16 @@
         <v>4</v>
       </c>
       <c r="J69" t="str">
-        <v>unidad</v>
+        <v>hoja</v>
       </c>
       <c r="K69" t="str">
         <v>H0005</v>
       </c>
       <c r="L69" s="2">
-        <v>10229.2902</v>
+        <v>2045.858</v>
       </c>
       <c r="M69" s="2">
-        <v>40917.16</v>
+        <v>8183.43</v>
       </c>
       <c r="N69" t="str">
         <v/>
@@ -8804,16 +8954,16 @@
         <v>4</v>
       </c>
       <c r="J70" t="str">
-        <v>unidad</v>
+        <v>hoja</v>
       </c>
       <c r="K70" t="str">
         <v>H0020</v>
       </c>
       <c r="L70" s="2">
-        <v>12026.9205</v>
+        <v>2405.3841</v>
       </c>
       <c r="M70" s="2">
-        <v>48107.68</v>
+        <v>9621.54</v>
       </c>
       <c r="N70" t="str">
         <v/>
@@ -9506,16 +9656,16 @@
         <v>2</v>
       </c>
       <c r="J85" t="str">
-        <v>unidad</v>
+        <v>hoja</v>
       </c>
       <c r="K85" t="str">
         <v>H0005</v>
       </c>
       <c r="L85" s="2">
-        <v>10229.2902</v>
+        <v>2045.858</v>
       </c>
       <c r="M85" s="2">
-        <v>20458.58</v>
+        <v>4091.72</v>
       </c>
       <c r="N85" t="str">
         <v/>
@@ -10226,7 +10376,7 @@
         <v>1</v>
       </c>
       <c r="J100" t="str">
-        <v>unidad</v>
+        <v>metro</v>
       </c>
       <c r="K100" t="str">
         <v>C0001</v>
@@ -13606,7 +13756,7 @@
         <v>1</v>
       </c>
       <c r="J170" t="str">
-        <v>unidad</v>
+        <v>metro</v>
       </c>
       <c r="K170" t="str">
         <v>C0001</v>
@@ -14488,16 +14638,16 @@
         <v>1</v>
       </c>
       <c r="J188" t="str">
-        <v>unidad</v>
+        <v>hoja</v>
       </c>
       <c r="K188" t="str">
         <v>H0020</v>
       </c>
       <c r="L188" s="2">
-        <v>12026.9205</v>
+        <v>2405.3841</v>
       </c>
       <c r="M188" s="2">
-        <v>12026.92</v>
+        <v>2405.38</v>
       </c>
       <c r="N188" t="str">
         <v/>
@@ -14720,16 +14870,16 @@
         <v>1</v>
       </c>
       <c r="J193" t="str">
-        <v>unidad</v>
+        <v>hoja</v>
       </c>
       <c r="K193" t="str">
         <v>H0005</v>
       </c>
       <c r="L193" s="2">
-        <v>10229.2902</v>
+        <v>2045.858</v>
       </c>
       <c r="M193" s="2">
-        <v>10229.29</v>
+        <v>2045.86</v>
       </c>
       <c r="N193" t="str">
         <v/>
@@ -14770,16 +14920,16 @@
         <v>1</v>
       </c>
       <c r="J194" t="str">
-        <v>unidad</v>
+        <v>hoja</v>
       </c>
       <c r="K194" t="str">
         <v>H0003</v>
       </c>
       <c r="L194" s="2">
-        <v>10581.9804</v>
+        <v>2116.3961</v>
       </c>
       <c r="M194" s="2">
-        <v>10581.98</v>
+        <v>2116.4</v>
       </c>
       <c r="N194" t="str">
         <v/>
@@ -14958,16 +15108,16 @@
         <v>1</v>
       </c>
       <c r="J198" t="str">
-        <v>unidad</v>
+        <v>hoja</v>
       </c>
       <c r="K198" t="str">
         <v>H0010</v>
       </c>
       <c r="L198" s="2">
-        <v>10240.8866</v>
+        <v>2048.1773</v>
       </c>
       <c r="M198" s="2">
-        <v>10240.89</v>
+        <v>2048.18</v>
       </c>
       <c r="N198" t="str">
         <v/>
@@ -16722,7 +16872,7 @@
         <v>1</v>
       </c>
       <c r="J234" t="str">
-        <v>unidad</v>
+        <v>metro</v>
       </c>
       <c r="K234" t="str">
         <v>C0001</v>
@@ -17198,7 +17348,7 @@
         <v>1</v>
       </c>
       <c r="J244" t="str">
-        <v>unidad</v>
+        <v>metro</v>
       </c>
       <c r="K244" t="str">
         <v>C0001</v>
@@ -19784,7 +19934,7 @@
         <v>1</v>
       </c>
       <c r="J298" t="str">
-        <v>unidad</v>
+        <v>metro</v>
       </c>
       <c r="K298" t="str">
         <v>C0001</v>
@@ -19984,7 +20134,7 @@
         <v>1</v>
       </c>
       <c r="J302" t="str">
-        <v>unidad</v>
+        <v>metro</v>
       </c>
       <c r="K302" t="str">
         <v>C0001</v>
@@ -23188,16 +23338,16 @@
         <v>2</v>
       </c>
       <c r="J368" t="str">
-        <v>unidad</v>
+        <v>hoja</v>
       </c>
       <c r="K368" t="str">
         <v>H0020</v>
       </c>
       <c r="L368" s="2">
-        <v>12026.9205</v>
+        <v>2405.3841</v>
       </c>
       <c r="M368" s="2">
-        <v>24053.84</v>
+        <v>4810.77</v>
       </c>
       <c r="N368" t="str">
         <v/>
@@ -43244,7 +43394,7 @@
         <v>7</v>
       </c>
       <c r="J781" t="str">
-        <v>unidad</v>
+        <v>metro</v>
       </c>
       <c r="K781" t="str">
         <v>C0001</v>
@@ -46736,16 +46886,16 @@
         <v>4</v>
       </c>
       <c r="J853" t="str">
-        <v>unidad</v>
+        <v>hoja</v>
       </c>
       <c r="K853" t="str">
         <v>H0010</v>
       </c>
       <c r="L853" s="2">
-        <v>10240.8866</v>
+        <v>2048.1773</v>
       </c>
       <c r="M853" s="2">
-        <v>40963.55</v>
+        <v>8192.71</v>
       </c>
       <c r="N853" t="str">
         <v/>
@@ -52236,7 +52386,7 @@
         <v>7</v>
       </c>
       <c r="J966" t="str">
-        <v>unidad</v>
+        <v>metro</v>
       </c>
       <c r="K966" t="str">
         <v>C0001</v>
@@ -55840,16 +55990,16 @@
         <v>1</v>
       </c>
       <c r="J1040" t="str">
-        <v>unidad</v>
+        <v>hoja</v>
       </c>
       <c r="K1040" t="str">
         <v>H0010</v>
       </c>
       <c r="L1040" s="2">
-        <v>10240.8866</v>
+        <v>2048.1773</v>
       </c>
       <c r="M1040" s="2">
-        <v>10240.89</v>
+        <v>2048.18</v>
       </c>
       <c r="N1040" t="str">
         <v/>
@@ -55890,16 +56040,16 @@
         <v>1</v>
       </c>
       <c r="J1041" t="str">
-        <v>unidad</v>
+        <v>hoja</v>
       </c>
       <c r="K1041" t="str">
         <v>H0020</v>
       </c>
       <c r="L1041" s="2">
-        <v>12026.9205</v>
+        <v>2405.3841</v>
       </c>
       <c r="M1041" s="2">
-        <v>12026.92</v>
+        <v>2405.38</v>
       </c>
       <c r="N1041" t="str">
         <v/>
@@ -55940,16 +56090,16 @@
         <v>1</v>
       </c>
       <c r="J1042" t="str">
-        <v>unidad</v>
+        <v>hoja</v>
       </c>
       <c r="K1042" t="str">
         <v>H0005</v>
       </c>
       <c r="L1042" s="2">
-        <v>10229.2902</v>
+        <v>2045.858</v>
       </c>
       <c r="M1042" s="2">
-        <v>10229.29</v>
+        <v>2045.86</v>
       </c>
       <c r="N1042" t="str">
         <v/>
@@ -55990,16 +56140,16 @@
         <v>1</v>
       </c>
       <c r="J1043" t="str">
-        <v>unidad</v>
+        <v>hoja</v>
       </c>
       <c r="K1043" t="str">
         <v>H0003</v>
       </c>
       <c r="L1043" s="2">
-        <v>10581.9804</v>
+        <v>2116.3961</v>
       </c>
       <c r="M1043" s="2">
-        <v>10581.98</v>
+        <v>2116.4</v>
       </c>
       <c r="N1043" t="str">
         <v/>
@@ -63318,7 +63468,7 @@
         <v>5</v>
       </c>
       <c r="J1194" t="str">
-        <v>unidad</v>
+        <v>metro</v>
       </c>
       <c r="K1194" t="str">
         <v>C0001</v>
@@ -68098,7 +68248,7 @@
         <v>5</v>
       </c>
       <c r="J1292" t="str">
-        <v>unidad</v>
+        <v>metro</v>
       </c>
       <c r="K1292" t="str">
         <v>C0001</v>
@@ -71472,7 +71622,7 @@
         <v>5</v>
       </c>
       <c r="J1362" t="str">
-        <v>unidad</v>
+        <v>metro</v>
       </c>
       <c r="K1362" t="str">
         <v>C0001</v>
@@ -73976,7 +74126,7 @@
         <v>5</v>
       </c>
       <c r="J1414" t="str">
-        <v>unidad</v>
+        <v>metro</v>
       </c>
       <c r="K1414" t="str">
         <v>C0001</v>
@@ -76166,16 +76316,16 @@
         <v>3</v>
       </c>
       <c r="J1459" t="str">
-        <v>unidad</v>
+        <v>hoja</v>
       </c>
       <c r="K1459" t="str">
         <v>H0005</v>
       </c>
       <c r="L1459" s="2">
-        <v>10229.2902</v>
+        <v>2045.858</v>
       </c>
       <c r="M1459" s="2">
-        <v>30687.87</v>
+        <v>6137.57</v>
       </c>
       <c r="N1459" t="str">
         <v/>
@@ -77851,7 +78001,7 @@
         <v>337</v>
       </c>
       <c r="C3" s="2">
-        <v>2522390.81</v>
+        <v>2359386.54</v>
       </c>
       <c r="D3">
         <v>120</v>
@@ -77865,7 +78015,7 @@
         <v>369</v>
       </c>
       <c r="C4" s="2">
-        <v>1813990.9</v>
+        <v>1778380.97</v>
       </c>
       <c r="D4">
         <v>94</v>
@@ -77893,7 +78043,7 @@
         <v>63</v>
       </c>
       <c r="C6" s="2">
-        <v>213055.47</v>
+        <v>178592.21</v>
       </c>
       <c r="D6">
         <v>17</v>
@@ -78017,44 +78167,44 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Hojas caladora y serrucho</v>
+        <v>Mechas</v>
       </c>
       <c r="B7">
-        <v>16</v>
+        <v>95</v>
       </c>
       <c r="C7" s="2">
-        <v>291346.84</v>
+        <v>247414.19</v>
       </c>
       <c r="D7">
-        <v>2</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Mechas</v>
+        <v>EPP</v>
       </c>
       <c r="B8">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="C8" s="2">
-        <v>247414.19</v>
+        <v>196071.51</v>
       </c>
       <c r="D8">
-        <v>11</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>EPP</v>
+        <v>Hojas caladora y serrucho</v>
       </c>
       <c r="B9">
-        <v>88</v>
+        <v>16</v>
       </c>
       <c r="C9" s="2">
-        <v>196071.51</v>
+        <v>58269.38</v>
       </c>
       <c r="D9">
-        <v>34</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -78195,7 +78345,7 @@
         <v>36</v>
       </c>
       <c r="C6" s="2">
-        <v>505457.02</v>
+        <v>472686.18</v>
       </c>
       <c r="D6">
         <v>13</v>
@@ -78217,30 +78367,30 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Galeano Caceres Willian Ivan</v>
+        <v>Indaburu Daniel Norberto</v>
       </c>
       <c r="B8">
-        <v>52</v>
+        <v>28</v>
       </c>
       <c r="C8" s="2">
-        <v>276273.28</v>
+        <v>265211.54</v>
       </c>
       <c r="D8">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Indaburu Daniel Norberto</v>
+        <v>Galeano Caceres Willian Ivan</v>
       </c>
       <c r="B9">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="C9" s="2">
-        <v>265211.54</v>
+        <v>217259.72</v>
       </c>
       <c r="D9">
-        <v>12</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10">
@@ -78307,7 +78457,7 @@
         <v>55</v>
       </c>
       <c r="C14" s="2">
-        <v>142065.98</v>
+        <v>125699.12</v>
       </c>
       <c r="D14">
         <v>15</v>
@@ -78315,167 +78465,167 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Gavilan Carlos Eloy</v>
+        <v>Salamonini Angel Humberto</v>
       </c>
       <c r="B15">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="C15" s="2">
-        <v>133089.18</v>
+        <v>102643.48</v>
       </c>
       <c r="D15">
-        <v>18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Montesano Maximiliano</v>
+        <v>Gavilan Carlos Eloy</v>
       </c>
       <c r="B16">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="C16" s="2">
-        <v>111593.26</v>
+        <v>98625.92</v>
       </c>
       <c r="D16">
-        <v>7</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Salamonini Angel Humberto</v>
+        <v>Zatta Lucas</v>
       </c>
       <c r="B17">
-        <v>12</v>
+        <v>37</v>
       </c>
       <c r="C17" s="2">
-        <v>102643.48</v>
+        <v>87030.89</v>
       </c>
       <c r="D17">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Zatta Lucas</v>
+        <v>Maldonado Jose lino</v>
       </c>
       <c r="B18">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="C18" s="2">
-        <v>87030.89</v>
+        <v>73984.1</v>
       </c>
       <c r="D18">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Maldonado Jose lino</v>
+        <v>Martinez Leandro Agustin</v>
       </c>
       <c r="B19">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="C19" s="2">
-        <v>73984.1</v>
+        <v>64453.96</v>
       </c>
       <c r="D19">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Martinez Leandro Agustin</v>
+        <v>Plaza Mauro</v>
       </c>
       <c r="B20">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="C20" s="2">
-        <v>64453.96</v>
+        <v>61059.06</v>
       </c>
       <c r="D20">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Plaza Mauro</v>
+        <v>Dure Franco Alejandro</v>
       </c>
       <c r="B21">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="C21" s="2">
-        <v>61059.06</v>
+        <v>60237.72</v>
       </c>
       <c r="D21">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Dure Franco Alejandro</v>
+        <v>Romero Tomas Ariel</v>
       </c>
       <c r="B22">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C22" s="2">
-        <v>60237.72</v>
+        <v>56621.18</v>
       </c>
       <c r="D22">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Romero Tomas Ariel</v>
+        <v>Chasco Marcos Eli</v>
       </c>
       <c r="B23">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C23" s="2">
-        <v>56621.18</v>
+        <v>50948.28</v>
       </c>
       <c r="D23">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Chasco Marcos Eli</v>
+        <v>Frias Gaston Dario</v>
       </c>
       <c r="B24">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C24" s="2">
-        <v>50948.28</v>
+        <v>44670.32</v>
       </c>
       <c r="D24">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Frias Gaston Dario</v>
+        <v>Orlando Jeremias David</v>
       </c>
       <c r="B25">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C25" s="2">
-        <v>44670.32</v>
+        <v>43945.23</v>
       </c>
       <c r="D25">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Orlando Jeremias David</v>
+        <v>Trejo Pablo Gaston</v>
       </c>
       <c r="B26">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C26" s="2">
-        <v>43945.23</v>
+        <v>43458.84</v>
       </c>
       <c r="D26">
         <v>3</v>
@@ -78483,16 +78633,16 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Trejo Pablo Gaston</v>
+        <v>Montesano Maximiliano</v>
       </c>
       <c r="B27">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C27" s="2">
-        <v>43458.84</v>
+        <v>40373.39</v>
       </c>
       <c r="D27">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="28">
@@ -78539,27 +78689,27 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Romero Alan</v>
+        <v>Metini Gustavo</v>
       </c>
       <c r="B31">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C31" s="2">
-        <v>32613.66</v>
+        <v>30595.66</v>
       </c>
       <c r="D31">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Metini Gustavo</v>
+        <v>Montesano Tobias Emanuel</v>
       </c>
       <c r="B32">
         <v>7</v>
       </c>
       <c r="C32" s="2">
-        <v>30595.66</v>
+        <v>29844.73</v>
       </c>
       <c r="D32">
         <v>2</v>
@@ -78567,100 +78717,100 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Montesano Tobias Emanuel</v>
+        <v>Gaona Juan Carlos</v>
       </c>
       <c r="B33">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="C33" s="2">
-        <v>29844.73</v>
+        <v>27256.97</v>
       </c>
       <c r="D33">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Gaona Juan Carlos</v>
+        <v>Cristaldo Raul Oscar</v>
       </c>
       <c r="B34">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="C34" s="2">
-        <v>27256.97</v>
+        <v>25290.75</v>
       </c>
       <c r="D34">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Cristaldo Raul Oscar</v>
+        <v>Iturrieta Ian Nicolas</v>
       </c>
       <c r="B35">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C35" s="2">
-        <v>25290.75</v>
+        <v>23868</v>
       </c>
       <c r="D35">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Iturrieta Ian Nicolas</v>
+        <v>Benitez Servin Bruno Francisco</v>
       </c>
       <c r="B36">
         <v>10</v>
       </c>
       <c r="C36" s="2">
-        <v>23868</v>
+        <v>17540.33</v>
       </c>
       <c r="D36">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Benitez Servin Bruno Francisco</v>
+        <v>Salazar Matias Ezequiel</v>
       </c>
       <c r="B37">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C37" s="2">
-        <v>17540.33</v>
+        <v>15261.4</v>
       </c>
       <c r="D37">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Salazar Matias Ezequiel</v>
+        <v>Moreno Claudio</v>
       </c>
       <c r="B38">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C38" s="2">
-        <v>15261.4</v>
+        <v>13475.13</v>
       </c>
       <c r="D38">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Moreno Claudio</v>
+        <v>Romero Alan</v>
       </c>
       <c r="B39">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C39" s="2">
-        <v>13475.13</v>
+        <v>13370.59</v>
       </c>
       <c r="D39">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
@@ -78921,30 +79071,30 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>52-26</v>
+        <v>37-39/40/41/42</v>
       </c>
       <c r="B8">
-        <v>110</v>
+        <v>22</v>
       </c>
       <c r="C8" s="2">
-        <v>426149.72</v>
+        <v>388559.23</v>
       </c>
       <c r="D8">
-        <v>34</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>37-39/40/41/42</v>
+        <v>52-26</v>
       </c>
       <c r="B9">
-        <v>22</v>
+        <v>110</v>
       </c>
       <c r="C9" s="2">
-        <v>388559.23</v>
+        <v>367136.16</v>
       </c>
       <c r="D9">
-        <v>6</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10">
@@ -78955,7 +79105,7 @@
         <v>52</v>
       </c>
       <c r="C10" s="2">
-        <v>382594.04</v>
+        <v>366227.18</v>
       </c>
       <c r="D10">
         <v>19</v>
@@ -78963,30 +79113,30 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>52-24</v>
+        <v>52-23</v>
       </c>
       <c r="B11">
-        <v>99</v>
+        <v>69</v>
       </c>
       <c r="C11" s="2">
-        <v>342299.57</v>
+        <v>333405.27</v>
       </c>
       <c r="D11">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>52-23</v>
+        <v>52-24</v>
       </c>
       <c r="B12">
-        <v>69</v>
+        <v>99</v>
       </c>
       <c r="C12" s="2">
-        <v>333405.27</v>
+        <v>307836.31</v>
       </c>
       <c r="D12">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13">
@@ -79033,55 +79183,55 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>64-21</v>
+        <v>37-42</v>
       </c>
       <c r="B16">
-        <v>56</v>
+        <v>32</v>
       </c>
       <c r="C16" s="2">
-        <v>256486.21</v>
+        <v>220166.19</v>
       </c>
       <c r="D16">
-        <v>18</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>37-42</v>
+        <v>PINTURA</v>
       </c>
       <c r="B17">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C17" s="2">
-        <v>252937.03</v>
+        <v>220142.82</v>
       </c>
       <c r="D17">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>PINTURA</v>
+        <v>K55</v>
       </c>
       <c r="B18">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C18" s="2">
-        <v>220142.82</v>
+        <v>201103.38</v>
       </c>
       <c r="D18">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>K55</v>
+        <v>52</v>
       </c>
       <c r="B19">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="C19" s="2">
-        <v>201103.38</v>
+        <v>189114.83</v>
       </c>
       <c r="D19">
         <v>2</v>
@@ -79089,16 +79239,16 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>52</v>
+        <v>64-21</v>
       </c>
       <c r="B20">
-        <v>17</v>
+        <v>56</v>
       </c>
       <c r="C20" s="2">
-        <v>189114.83</v>
+        <v>185266.34</v>
       </c>
       <c r="D20">
-        <v>2</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21">
@@ -79179,7 +79329,7 @@
         <v>27</v>
       </c>
       <c r="C26" s="2">
-        <v>68210.5</v>
+        <v>48967.43</v>
       </c>
       <c r="D26">
         <v>5</v>
@@ -79527,198 +79677,198 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>2026-08 · Hojas caladora y serrucho</v>
+        <v>2026-08 · Limpieza y descarte</v>
       </c>
       <c r="B16">
-        <v>9</v>
+        <v>59</v>
       </c>
       <c r="C16" s="2">
-        <v>176616.34</v>
+        <v>164620</v>
       </c>
       <c r="D16">
-        <v>1</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>2026-08 · Limpieza y descarte</v>
+        <v>2026-09 · EPP</v>
       </c>
       <c r="B17">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="C17" s="2">
-        <v>164620</v>
+        <v>121519.16</v>
       </c>
       <c r="D17">
-        <v>32</v>
+        <v>10</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>2026-09 · EPP</v>
+        <v>2026-08 · Pintura y aplicación</v>
       </c>
       <c r="B18">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C18" s="2">
-        <v>121519.16</v>
+        <v>64848.45</v>
       </c>
       <c r="D18">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>2026-09 · Hojas caladora y serrucho</v>
+        <v>2026-10 · EPP</v>
       </c>
       <c r="B19">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="C19" s="2">
-        <v>84042.63</v>
+        <v>48104.5</v>
       </c>
       <c r="D19">
-        <v>1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>2026-08 · Pintura y aplicación</v>
+        <v>2026-08 · Mechas</v>
       </c>
       <c r="B20">
         <v>35</v>
       </c>
       <c r="C20" s="2">
-        <v>64848.45</v>
+        <v>41576.76</v>
       </c>
       <c r="D20">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>2026-10 · EPP</v>
+        <v>2026-08 · Hojas caladora y serrucho</v>
       </c>
       <c r="B21">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="C21" s="2">
-        <v>48104.5</v>
+        <v>35323.28</v>
       </c>
       <c r="D21">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>2026-08 · Mechas</v>
+        <v>2026-09 · Herramientas menores</v>
       </c>
       <c r="B22">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="C22" s="2">
-        <v>41576.76</v>
+        <v>32821.27</v>
       </c>
       <c r="D22">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>2026-09 · Herramientas menores</v>
+        <v>2026-08 · EPP</v>
       </c>
       <c r="B23">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="C23" s="2">
-        <v>32821.27</v>
+        <v>26447.85</v>
       </c>
       <c r="D23">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>2026-10 · Hojas caladora y serrucho</v>
+        <v>2026-10 · Mechas</v>
       </c>
       <c r="B24">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C24" s="2">
-        <v>30687.87</v>
+        <v>24908.32</v>
       </c>
       <c r="D24">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>2026-08 · EPP</v>
+        <v>2026-08 · Herramientas menores</v>
       </c>
       <c r="B25">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="C25" s="2">
-        <v>26447.85</v>
+        <v>17131.87</v>
       </c>
       <c r="D25">
-        <v>14</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>2026-10 · Mechas</v>
+        <v>2026-09 · Hojas caladora y serrucho</v>
       </c>
       <c r="B26">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C26" s="2">
-        <v>24908.32</v>
+        <v>16808.53</v>
       </c>
       <c r="D26">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>2026-08 · Herramientas menores</v>
+        <v>2026-08 · Fijaciones</v>
       </c>
       <c r="B27">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="C27" s="2">
-        <v>17131.87</v>
+        <v>14597.66</v>
       </c>
       <c r="D27">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>2026-08 · Fijaciones</v>
+        <v>2026-09 · Fijaciones</v>
       </c>
       <c r="B28">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="C28" s="2">
-        <v>14597.66</v>
+        <v>9655.5</v>
       </c>
       <c r="D28">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>2026-09 · Fijaciones</v>
+        <v>2026-10 · Hojas caladora y serrucho</v>
       </c>
       <c r="B29">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="C29" s="2">
-        <v>9655.5</v>
+        <v>6137.57</v>
       </c>
       <c r="D29">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -80736,7 +80886,7 @@
         <v>40</v>
       </c>
       <c r="F38" t="str">
-        <v>unidad</v>
+        <v>metro</v>
       </c>
       <c r="G38" s="2">
         <v>462800</v>
@@ -81408,10 +81558,10 @@
         <v>11</v>
       </c>
       <c r="F65" t="str">
-        <v>unidad</v>
+        <v>hoja</v>
       </c>
       <c r="G65" s="2">
-        <v>112522.19</v>
+        <v>22504.44</v>
       </c>
       <c r="H65" t="b">
         <v>1</v>
@@ -81564,10 +81714,10 @@
         <v>8</v>
       </c>
       <c r="F71" t="str">
-        <v>unidad</v>
+        <v>hoja</v>
       </c>
       <c r="G71" s="2">
-        <v>96215.36</v>
+        <v>19243.07</v>
       </c>
       <c r="H71" t="b">
         <v>1</v>
@@ -81812,10 +81962,10 @@
         <v>6</v>
       </c>
       <c r="F81" t="str">
-        <v>unidad</v>
+        <v>hoja</v>
       </c>
       <c r="G81" s="2">
-        <v>61445.33</v>
+        <v>12289.07</v>
       </c>
       <c r="H81" t="b">
         <v>1</v>
@@ -81988,10 +82138,10 @@
         <v>2</v>
       </c>
       <c r="F88" t="str">
-        <v>unidad</v>
+        <v>hoja</v>
       </c>
       <c r="G88" s="2">
-        <v>21163.96</v>
+        <v>4232.8</v>
       </c>
       <c r="H88" t="b">
         <v>1</v>

</xml_diff>